<commit_message>
Aggiornamento dati del 20/08/2026
</commit_message>
<xml_diff>
--- a/dati/Gestione.xlsx
+++ b/dati/Gestione.xlsx
@@ -36,354 +36,354 @@
     <t>Questo file e' la fonte unica dei dati del sito.</t>
   </si>
   <si>
+    <t>Dopo averlo modificato e SALVATO: doppio click su aggiorna.bat</t>
+  </si>
+  <si>
+    <t>Foglio</t>
+  </si>
+  <si>
+    <t>Allenatore</t>
+  </si>
+  <si>
+    <t>Anno</t>
+  </si>
+  <si>
+    <t>Squadra</t>
+  </si>
+  <si>
+    <t>Nome</t>
+  </si>
+  <si>
     <t>Giocatore</t>
   </si>
   <si>
-    <t>Allenatore</t>
-  </si>
-  <si>
-    <t>Squadra</t>
-  </si>
-  <si>
-    <t>Dopo averlo modificato e SALVATO: doppio click su aggiorna.bat</t>
+    <t>Tabella SQLite</t>
+  </si>
+  <si>
+    <t>Contenuto</t>
+  </si>
+  <si>
+    <t>AnagraficaSquadre</t>
+  </si>
+  <si>
+    <t>teams</t>
   </si>
   <si>
     <t>Mindo</t>
   </si>
   <si>
+    <t>Squadre e allenatori (qui stanno gli ID)</t>
+  </si>
+  <si>
     <t>Chentus</t>
   </si>
   <si>
-    <t>Foglio</t>
+    <t>CambioNome</t>
+  </si>
+  <si>
+    <t>cambio_nome</t>
+  </si>
+  <si>
+    <t>Nome della squadra per anno</t>
   </si>
   <si>
     <t>Alessio Cocchieri &amp; Febio</t>
   </si>
   <si>
+    <t>Contratti</t>
+  </si>
+  <si>
+    <t>contracts + players</t>
+  </si>
+  <si>
     <t>MALLOREDDUS FC</t>
   </si>
   <si>
+    <t>Contratti di riconferma</t>
+  </si>
+  <si>
+    <t>Svincoli</t>
+  </si>
+  <si>
+    <t>PietroPJ</t>
+  </si>
+  <si>
+    <t>contract_releases</t>
+  </si>
+  <si>
     <t>AnnoNascita</t>
   </si>
   <si>
-    <t>Tabella SQLite</t>
+    <t>Sporting Garra</t>
+  </si>
+  <si>
+    <t>Svincoli: storico e penali</t>
   </si>
   <si>
     <t>IDSquadra</t>
   </si>
   <si>
-    <t>PietroPJ</t>
-  </si>
-  <si>
-    <t>Contenuto</t>
-  </si>
-  <si>
-    <t>Sporting Garra</t>
+    <t>Classifiche</t>
   </si>
   <si>
     <t>AnnoInizio</t>
   </si>
   <si>
+    <t>Max Allegri</t>
+  </si>
+  <si>
+    <t>season_rankings</t>
+  </si>
+  <si>
+    <t>Whiteam FC</t>
+  </si>
+  <si>
+    <t>Classifica di campionato</t>
+  </si>
+  <si>
+    <t>Coppa</t>
+  </si>
+  <si>
+    <t>Fil e Pacciansss &amp; sono innocenti</t>
+  </si>
+  <si>
+    <t>coppa</t>
+  </si>
+  <si>
+    <t>TurettaEPacciani FC</t>
+  </si>
+  <si>
+    <t>Podio della coppa</t>
+  </si>
+  <si>
+    <t>CreditiAsta</t>
+  </si>
+  <si>
+    <t>credit_residual</t>
+  </si>
+  <si>
+    <t>Alessio Bruni</t>
+  </si>
+  <si>
+    <t>Crediti avanzati a fine stagione</t>
+  </si>
+  <si>
+    <t>Nkunku Settete</t>
+  </si>
+  <si>
+    <t>CreditiAnnoNuovo</t>
+  </si>
+  <si>
     <t>PrezzoAcquisto</t>
   </si>
   <si>
-    <t>AnagraficaSquadre</t>
+    <t>crediti_anno_nuovo</t>
+  </si>
+  <si>
+    <t>deiu &amp; Bep</t>
+  </si>
+  <si>
+    <t>Budget della stagione nuova</t>
   </si>
   <si>
     <t>Attivo</t>
   </si>
   <si>
-    <t>teams</t>
-  </si>
-  <si>
-    <t>Max Allegri</t>
-  </si>
-  <si>
-    <t>Squadre e allenatori (qui stanno gli ID)</t>
-  </si>
-  <si>
-    <t>Anno</t>
+    <t>Mapi Group</t>
+  </si>
+  <si>
+    <t>FOGLIO CONTRATTI</t>
+  </si>
+  <si>
+    <t>CariBam &amp; sickroul</t>
+  </si>
+  <si>
+    <t>nome del calciatore, scritto per esteso</t>
   </si>
   <si>
     <t>Alvarez</t>
   </si>
   <si>
-    <t>Whiteam FC</t>
-  </si>
-  <si>
-    <t>CambioNome</t>
-  </si>
-  <si>
-    <t>Nome</t>
-  </si>
-  <si>
-    <t>cambio_nome</t>
-  </si>
-  <si>
-    <t>Nome della squadra per anno</t>
-  </si>
-  <si>
-    <t>Fil e Pacciansss &amp; sono innocenti</t>
-  </si>
-  <si>
-    <t>TurettaEPacciani FC</t>
-  </si>
-  <si>
-    <t>Contratti</t>
-  </si>
-  <si>
-    <t>contracts + players</t>
-  </si>
-  <si>
-    <t>Alessio Bruni</t>
-  </si>
-  <si>
-    <t>Contratti di riconferma</t>
-  </si>
-  <si>
-    <t>Nkunku Settete</t>
+    <t>Roul e il socio</t>
+  </si>
+  <si>
+    <t>solo l'anno: da qui dipende la categoria A/B/C</t>
+  </si>
+  <si>
+    <t>Luca baffi e tabacchi</t>
+  </si>
+  <si>
+    <t>ID come in AnagraficaSquadre</t>
+  </si>
+  <si>
+    <t>Compagnia Ascolana Sigari</t>
+  </si>
+  <si>
+    <t>anno della riconferma</t>
+  </si>
+  <si>
+    <t>mister zeman</t>
+  </si>
+  <si>
+    <t>prezzo pagato all'asta: non cambia mai</t>
+  </si>
+  <si>
+    <t>1 se in corso, 0 se chiuso</t>
+  </si>
+  <si>
+    <t>ANNO FINE NON SI SCRIVE</t>
+  </si>
+  <si>
+    <t>e' sempre AnnoInizio + 3 (regolamento par. 1)</t>
   </si>
   <si>
     <t>Perin</t>
   </si>
   <si>
-    <t>Svincoli</t>
-  </si>
-  <si>
-    <t>contract_releases</t>
-  </si>
-  <si>
-    <t>Svincoli: storico e penali</t>
-  </si>
-  <si>
-    <t>deiu &amp; Bep</t>
-  </si>
-  <si>
-    <t>Mapi Group</t>
-  </si>
-  <si>
-    <t>Classifiche</t>
+    <t>FOGLIO SVINCOLI</t>
+  </si>
+  <si>
+    <t>Tridente demoniaco</t>
+  </si>
+  <si>
+    <t>stesso nome scritto in Contratti</t>
+  </si>
+  <si>
+    <t>la squadra che lo svincola</t>
+  </si>
+  <si>
+    <t>AnnoSvincolo</t>
+  </si>
+  <si>
+    <t>anno in cui viene svincolato</t>
+  </si>
+  <si>
+    <t>Penale</t>
   </si>
   <si>
     <t>Conti</t>
   </si>
   <si>
-    <t>season_rankings</t>
-  </si>
-  <si>
-    <t>Classifica di campionato</t>
-  </si>
-  <si>
-    <t>CariBam &amp; sickroul</t>
-  </si>
-  <si>
-    <t>Roul e il socio</t>
+    <t>LASCIALA VUOTA: la calcola il sistema.</t>
+  </si>
+  <si>
+    <t>Compilala solo per forzare un valore diverso.</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>motivo, facoltativo</t>
+  </si>
+  <si>
+    <t>QUANDO SVINCOLI UN GIOCATORE</t>
+  </si>
+  <si>
+    <t>1. Aggiungi la riga qui in Svincoli</t>
   </si>
   <si>
     <t>Donati</t>
   </si>
   <si>
-    <t>Coppa</t>
-  </si>
-  <si>
-    <t>Luca baffi e tabacchi</t>
-  </si>
-  <si>
-    <t>coppa</t>
-  </si>
-  <si>
-    <t>Compagnia Ascolana Sigari</t>
-  </si>
-  <si>
-    <t>Podio della coppa</t>
+    <t>2. Metti Attivo = 0 nella sua riga di Contratti</t>
+  </si>
+  <si>
+    <t>La penale viene tolta dai crediti dell'asta successiva.</t>
+  </si>
+  <si>
+    <t>CATEGORIE (sull'anno di riferimento)</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>eta' &lt;= 21</t>
+  </si>
+  <si>
+    <t>illimitati</t>
+  </si>
+  <si>
+    <t>B</t>
   </si>
   <si>
     <t>Ferraro</t>
   </si>
   <si>
-    <t>CreditiAsta</t>
-  </si>
-  <si>
-    <t>mister zeman</t>
-  </si>
-  <si>
-    <t>credit_residual</t>
-  </si>
-  <si>
-    <t>Tridente demoniaco</t>
-  </si>
-  <si>
-    <t>Crediti avanzati a fine stagione</t>
+    <t>eta' &lt;= 25</t>
+  </si>
+  <si>
+    <t>nessun limite proprio, ma A+B &lt;= 6</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>oltre i 25</t>
+  </si>
+  <si>
+    <t>massimo 3</t>
+  </si>
+  <si>
+    <t>CREDITI DELLA STAGIONE NUOVA</t>
   </si>
   <si>
     <t>Gatti</t>
   </si>
   <si>
-    <t>CreditiAnnoNuovo</t>
-  </si>
-  <si>
-    <t>crediti_anno_nuovo</t>
+    <t>Non si compilano a mano.</t>
+  </si>
+  <si>
+    <t>strumenti\calcola_crediti.py li calcola</t>
   </si>
   <si>
     <t>Moretti</t>
   </si>
   <si>
-    <t>Budget della stagione nuova</t>
-  </si>
-  <si>
-    <t>FOGLIO CONTRATTI</t>
-  </si>
-  <si>
     <t>Rinaldi</t>
   </si>
   <si>
-    <t>nome del calciatore, scritto per esteso</t>
-  </si>
-  <si>
     <t>Santoro</t>
   </si>
   <si>
-    <t>solo l'anno: da qui dipende la categoria A/B/C</t>
-  </si>
-  <si>
     <t>Lombardi</t>
   </si>
   <si>
-    <t>ID come in AnagraficaSquadre</t>
-  </si>
-  <si>
-    <t>anno della riconferma</t>
-  </si>
-  <si>
     <t>Ricci</t>
   </si>
   <si>
-    <t>prezzo pagato all'asta: non cambia mai</t>
-  </si>
-  <si>
     <t>Marino</t>
   </si>
   <si>
-    <t>1 se in corso, 0 se chiuso</t>
-  </si>
-  <si>
     <t>Baggio</t>
   </si>
   <si>
-    <t>ANNO FINE NON SI SCRIVE</t>
-  </si>
-  <si>
-    <t>e' sempre AnnoInizio + 3 (regolamento par. 1)</t>
-  </si>
-  <si>
     <t>Greco</t>
   </si>
   <si>
-    <t>FOGLIO SVINCOLI</t>
-  </si>
-  <si>
     <t>Romano</t>
   </si>
   <si>
-    <t>stesso nome scritto in Contratti</t>
-  </si>
-  <si>
     <t>Martini</t>
   </si>
   <si>
-    <t>la squadra che lo svincola</t>
-  </si>
-  <si>
-    <t>AnnoSvincolo</t>
-  </si>
-  <si>
     <t>Costa</t>
   </si>
   <si>
-    <t>anno in cui viene svincolato</t>
-  </si>
-  <si>
-    <t>Penale</t>
-  </si>
-  <si>
-    <t>LASCIALA VUOTA: la calcola il sistema.</t>
-  </si>
-  <si>
     <t>Serra</t>
   </si>
   <si>
-    <t>Compilala solo per forzare un valore diverso.</t>
-  </si>
-  <si>
     <t>Pellegrini</t>
   </si>
   <si>
-    <t>Note</t>
-  </si>
-  <si>
-    <t>motivo, facoltativo</t>
-  </si>
-  <si>
-    <t>QUANDO SVINCOLI UN GIOCATORE</t>
-  </si>
-  <si>
     <t>Vitale</t>
   </si>
   <si>
-    <t>1. Aggiungi la riga qui in Svincoli</t>
-  </si>
-  <si>
     <t>Colombo</t>
   </si>
   <si>
-    <t>2. Metti Attivo = 0 nella sua riga di Contratti</t>
-  </si>
-  <si>
-    <t>La penale viene tolta dai crediti dell'asta successiva.</t>
-  </si>
-  <si>
     <t>Esposito</t>
   </si>
   <si>
-    <t>CATEGORIE (sull'anno di riferimento)</t>
-  </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
-    <t>eta' &lt;= 21</t>
-  </si>
-  <si>
-    <t>illimitati</t>
-  </si>
-  <si>
-    <t>B</t>
-  </si>
-  <si>
-    <t>eta' &lt;= 25</t>
-  </si>
-  <si>
-    <t>nessun limite proprio, ma A+B &lt;= 6</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>oltre i 25</t>
-  </si>
-  <si>
-    <t>massimo 3</t>
-  </si>
-  <si>
-    <t>CREDITI DELLA STAGIONE NUOVA</t>
-  </si>
-  <si>
-    <t>Non si compilano a mano.</t>
-  </si>
-  <si>
-    <t>strumenti\calcola_crediti.py li calcola</t>
-  </si>
-  <si>
     <t>Posizione</t>
   </si>
   <si>
@@ -405,10 +405,10 @@
     <t>Crediti da Punteggio</t>
   </si>
   <si>
+    <t>Crediti per Anno Nuovo</t>
+  </si>
+  <si>
     <t>Categoria</t>
-  </si>
-  <si>
-    <t>Crediti per Anno Nuovo</t>
   </si>
   <si>
     <t>Valore</t>
@@ -484,14 +484,14 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11.0"/>
-      <color rgb="FFFFFFFF"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <color theme="1"/>
+      <b/>
+      <sz val="11.0"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
@@ -551,21 +551,21 @@
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -829,298 +829,298 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="s">
-        <v>6</v>
+      <c r="A4" s="2" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="s">
+      <c r="C17" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C8" s="3" t="s">
+      <c r="C18" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="C13" s="3" t="s">
+      <c r="C19" s="2" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="3" t="s">
+    <row r="20">
+      <c r="A20" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B14" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="C14" s="3" t="s">
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="5" t="s">
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="2" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>82</v>
+      <c r="C23" s="2" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1"/>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="5" t="s">
-        <v>84</v>
+      <c r="A25" s="4" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>86</v>
+      <c r="A26" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>88</v>
+      <c r="A27" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>91</v>
+      <c r="A28" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>93</v>
+      <c r="A29" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="C30" s="3" t="s">
-        <v>95</v>
+      <c r="C30" s="2" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="C31" s="3" t="s">
-        <v>98</v>
+      <c r="A31" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1"/>
     <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="5" t="s">
-        <v>99</v>
+      <c r="A33" s="4" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="3" t="s">
-        <v>101</v>
+      <c r="A34" s="2" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
-      <c r="A35" s="3" t="s">
-        <v>103</v>
+      <c r="A35" s="2" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
-      <c r="A36" s="3" t="s">
-        <v>104</v>
+      <c r="A36" s="2" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1"/>
     <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="5" t="s">
-        <v>106</v>
+      <c r="A38" s="4" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
-      <c r="A39" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="C39" s="3" t="s">
-        <v>109</v>
+      <c r="A39" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
-      <c r="A40" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="C40" s="3" t="s">
-        <v>112</v>
+      <c r="A40" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
-      <c r="A41" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="B41" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="C41" s="3" t="s">
-        <v>115</v>
+      <c r="A41" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1"/>
     <row r="43" ht="15.75" customHeight="1">
-      <c r="A43" s="5" t="s">
-        <v>116</v>
+      <c r="A43" s="4" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
-      <c r="A44" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="C44" s="3" t="s">
-        <v>118</v>
+      <c r="A44" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1"/>
@@ -2105,7 +2105,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>119</v>
@@ -2114,7 +2114,7 @@
         <v>128</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="E1" s="8" t="s">
         <v>129</v>
@@ -2124,321 +2124,321 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="2">
         <v>1000.0</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2" s="2">
         <v>2999.0</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="2" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="2">
         <v>950.0</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E3" s="2">
         <v>2999.0</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="2" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="2">
         <v>1100.0</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="2">
         <v>2999.0</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="2" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="2">
         <v>900.0</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5" s="2">
         <v>2999.0</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="2" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="2">
         <v>1.0</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="2">
         <v>25.0</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E6" s="3">
+      <c r="E6" s="2">
         <v>2999.0</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="2" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7" s="2">
         <v>2.0</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="2">
         <v>15.0</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E7" s="3">
+      <c r="E7" s="2">
         <v>2999.0</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="2" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B8" s="2">
         <v>3.0</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="2">
         <v>10.0</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E8" s="3">
+      <c r="E8" s="2">
         <v>2999.0</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="F8" s="2" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="B9" s="3">
+      <c r="B9" s="2">
         <v>4.0</v>
       </c>
-      <c r="C9" s="3">
+      <c r="C9" s="2">
         <v>5.0</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E9" s="3">
+      <c r="E9" s="2">
         <v>2999.0</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="F9" s="2" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="B10" s="3">
+      <c r="B10" s="2">
         <v>5.0</v>
       </c>
-      <c r="C10" s="3">
+      <c r="C10" s="2">
         <v>0.0</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E10" s="3">
+      <c r="E10" s="2">
         <v>2999.0</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="F10" s="2" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="B11" s="3">
+      <c r="B11" s="2">
         <v>6.0</v>
       </c>
-      <c r="C11" s="3">
+      <c r="C11" s="2">
         <v>0.0</v>
       </c>
-      <c r="D11" s="3">
+      <c r="D11" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E11" s="3">
+      <c r="E11" s="2">
         <v>2999.0</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="F11" s="2" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="B12" s="3">
+      <c r="B12" s="2">
         <v>7.0</v>
       </c>
-      <c r="C12" s="3">
+      <c r="C12" s="2">
         <v>-5.0</v>
       </c>
-      <c r="D12" s="3">
+      <c r="D12" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E12" s="3">
+      <c r="E12" s="2">
         <v>2999.0</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="F12" s="2" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="B13" s="3">
+      <c r="B13" s="2">
         <v>8.0</v>
       </c>
-      <c r="C13" s="3">
+      <c r="C13" s="2">
         <v>-10.0</v>
       </c>
-      <c r="D13" s="3">
+      <c r="D13" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E13" s="3">
+      <c r="E13" s="2">
         <v>2999.0</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="F13" s="2" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="B14" s="3">
+      <c r="B14" s="2">
         <v>9.0</v>
       </c>
-      <c r="C14" s="3">
+      <c r="C14" s="2">
         <v>-15.0</v>
       </c>
-      <c r="D14" s="3">
+      <c r="D14" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E14" s="3">
+      <c r="E14" s="2">
         <v>2999.0</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="F14" s="2" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="B15" s="3">
+      <c r="B15" s="2">
         <v>10.0</v>
       </c>
-      <c r="C15" s="3">
+      <c r="C15" s="2">
         <v>-20.0</v>
       </c>
-      <c r="D15" s="3">
+      <c r="D15" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E15" s="3">
+      <c r="E15" s="2">
         <v>2999.0</v>
       </c>
-      <c r="F15" s="3" t="s">
+      <c r="F15" s="2" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="C16" s="3">
+      <c r="C16" s="2">
         <v>10.0</v>
       </c>
-      <c r="D16" s="3">
+      <c r="D16" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E16" s="3">
+      <c r="E16" s="2">
         <v>2999.0</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="F16" s="2" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="C17" s="3">
+      <c r="A17" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17" s="2">
         <v>10.0</v>
       </c>
-      <c r="D17" s="3">
+      <c r="D17" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E17" s="3">
+      <c r="E17" s="2">
         <v>2999.0</v>
       </c>
-      <c r="F17" s="3" t="s">
+      <c r="F17" s="2" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="C18" s="3">
+      <c r="C18" s="2">
         <v>50.0</v>
       </c>
-      <c r="D18" s="3">
+      <c r="D18" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E18" s="3">
+      <c r="E18" s="2">
         <v>2999.0</v>
       </c>
-      <c r="F18" s="3" t="s">
+      <c r="F18" s="2" t="s">
         <v>145</v>
       </c>
     </row>
@@ -3444,124 +3444,124 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>5</v>
       </c>
+      <c r="C1" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="3">
+      <c r="A2" s="2">
         <v>1.0</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>8</v>
+      <c r="B2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3">
+      <c r="A3" s="2">
         <v>2.0</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>11</v>
+      <c r="B3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3">
+      <c r="A4" s="2">
         <v>3.0</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>17</v>
+      <c r="B4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3">
+      <c r="A5" s="2">
         <v>4.0</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>27</v>
+      <c r="B5" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3">
+      <c r="A6" s="2">
         <v>5.0</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>33</v>
+      <c r="B6" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3">
+      <c r="A7" s="2">
         <v>6.0</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>38</v>
+      <c r="B7" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3">
+      <c r="A8" s="2">
         <v>7.0</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>44</v>
+      <c r="B8" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3">
+      <c r="A9" s="2">
         <v>8.0</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>50</v>
+      <c r="B9" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3">
+      <c r="A10" s="2">
         <v>9.0</v>
       </c>
-      <c r="B10" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>55</v>
+      <c r="B10" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3">
+      <c r="A11" s="2">
         <v>10.0</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>61</v>
+      <c r="B11" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -4565,124 +4565,124 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="B1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="B2" s="2">
+        <v>2026.0</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="B3" s="2">
+        <v>2026.0</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2">
+        <v>3.0</v>
+      </c>
+      <c r="B4" s="2">
+        <v>2026.0</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="3">
-        <v>1.0</v>
-      </c>
-      <c r="B2" s="3">
+    <row r="5">
+      <c r="A5" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="B5" s="2">
         <v>2026.0</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3">
-        <v>2.0</v>
-      </c>
-      <c r="B3" s="3">
+      <c r="C5" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2">
+        <v>5.0</v>
+      </c>
+      <c r="B6" s="2">
         <v>2026.0</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3">
-        <v>3.0</v>
-      </c>
-      <c r="B4" s="3">
+      <c r="C6" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2">
+        <v>6.0</v>
+      </c>
+      <c r="B7" s="2">
         <v>2026.0</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3">
-        <v>4.0</v>
-      </c>
-      <c r="B5" s="3">
+      <c r="C7" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2">
+        <v>7.0</v>
+      </c>
+      <c r="B8" s="2">
         <v>2026.0</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3">
-        <v>5.0</v>
-      </c>
-      <c r="B6" s="3">
+      <c r="C8" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2">
+        <v>8.0</v>
+      </c>
+      <c r="B9" s="2">
         <v>2026.0</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3">
-        <v>6.0</v>
-      </c>
-      <c r="B7" s="3">
+      <c r="C9" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2">
+        <v>9.0</v>
+      </c>
+      <c r="B10" s="2">
         <v>2026.0</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3">
-        <v>7.0</v>
-      </c>
-      <c r="B8" s="3">
+      <c r="C10" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2">
+        <v>10.0</v>
+      </c>
+      <c r="B11" s="2">
         <v>2026.0</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3">
-        <v>8.0</v>
-      </c>
-      <c r="B9" s="3">
-        <v>2026.0</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3">
-        <v>9.0</v>
-      </c>
-      <c r="B10" s="3">
-        <v>2026.0</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3">
-        <v>10.0</v>
-      </c>
-      <c r="B11" s="3">
-        <v>2026.0</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>61</v>
+      <c r="C11" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -5689,462 +5689,477 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>21</v>
+      <c r="A1" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="B2" s="3">
+        <v>58</v>
+      </c>
+      <c r="B2" s="2">
         <v>2006.0</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="2">
         <v>1.0</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2" s="2">
         <v>21.0</v>
       </c>
-      <c r="F2" s="3">
+      <c r="F2" s="2">
         <v>1.0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B3" s="3">
+        <v>70</v>
+      </c>
+      <c r="B3" s="2">
+        <v>2006.0</v>
+      </c>
+      <c r="C3" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="D3" s="2">
+        <v>2026.0</v>
+      </c>
+      <c r="E3" s="2">
+        <v>11.0</v>
+      </c>
+      <c r="F3" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="I3" s="2">
         <v>2003.0</v>
-      </c>
-      <c r="C3" s="3">
-        <v>1.0</v>
-      </c>
-      <c r="D3" s="3">
-        <v>2026.0</v>
-      </c>
-      <c r="E3" s="3">
-        <v>11.0</v>
-      </c>
-      <c r="F3" s="3">
-        <v>1.0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="B4" s="3">
+        <v>78</v>
+      </c>
+      <c r="B4" s="2">
+        <v>2006.0</v>
+      </c>
+      <c r="C4" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="D4" s="2">
+        <v>2026.0</v>
+      </c>
+      <c r="E4" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F4" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="I4" s="2">
         <v>1997.0</v>
-      </c>
-      <c r="C4" s="3">
-        <v>1.0</v>
-      </c>
-      <c r="D4" s="3">
-        <v>2026.0</v>
-      </c>
-      <c r="E4" s="3">
-        <v>24.0</v>
-      </c>
-      <c r="F4" s="3">
-        <v>1.0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="B5" s="3">
+        <v>85</v>
+      </c>
+      <c r="B5" s="2">
+        <v>2006.0</v>
+      </c>
+      <c r="C5" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="D5" s="2">
+        <v>2026.0</v>
+      </c>
+      <c r="E5" s="2">
+        <v>31.0</v>
+      </c>
+      <c r="F5" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="I5" s="2">
         <v>1996.0</v>
-      </c>
-      <c r="C5" s="3">
-        <v>1.0</v>
-      </c>
-      <c r="D5" s="3">
-        <v>2026.0</v>
-      </c>
-      <c r="E5" s="3">
-        <v>31.0</v>
-      </c>
-      <c r="F5" s="3">
-        <v>1.0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B6" s="3">
+        <v>93</v>
+      </c>
+      <c r="B6" s="2">
+        <v>2006.0</v>
+      </c>
+      <c r="C6" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="D6" s="2">
+        <v>2026.0</v>
+      </c>
+      <c r="E6" s="2">
+        <v>122.0</v>
+      </c>
+      <c r="F6" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="I6" s="2">
         <v>1996.0</v>
-      </c>
-      <c r="C6" s="3">
-        <v>1.0</v>
-      </c>
-      <c r="D6" s="3">
-        <v>2026.0</v>
-      </c>
-      <c r="E6" s="3">
-        <v>122.0</v>
-      </c>
-      <c r="F6" s="3">
-        <v>1.0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="B7" s="3">
+        <v>100</v>
+      </c>
+      <c r="B7" s="2">
+        <v>2006.0</v>
+      </c>
+      <c r="C7" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="D7" s="2">
+        <v>2026.0</v>
+      </c>
+      <c r="E7" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="F7" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="I7" s="2">
         <v>2001.0</v>
-      </c>
-      <c r="C7" s="3">
-        <v>1.0</v>
-      </c>
-      <c r="D7" s="3">
-        <v>2026.0</v>
-      </c>
-      <c r="E7" s="3">
-        <v>1.0</v>
-      </c>
-      <c r="F7" s="3">
-        <v>1.0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="B8" s="3">
+        <v>103</v>
+      </c>
+      <c r="B8" s="2">
         <v>2000.0</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="2">
         <v>4.0</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E8" s="3">
+      <c r="E8" s="2">
         <v>210.0</v>
       </c>
-      <c r="F8" s="3">
+      <c r="F8" s="2">
         <v>1.0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="B9" s="3">
+        <v>104</v>
+      </c>
+      <c r="B9" s="2">
         <v>1997.0</v>
       </c>
-      <c r="C9" s="3">
+      <c r="C9" s="2">
         <v>4.0</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E9" s="3">
+      <c r="E9" s="2">
         <v>95.0</v>
       </c>
-      <c r="F9" s="3">
+      <c r="F9" s="2">
         <v>1.0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="B10" s="3">
+        <v>105</v>
+      </c>
+      <c r="B10" s="2">
         <v>1999.0</v>
       </c>
-      <c r="C10" s="3">
+      <c r="C10" s="2">
         <v>4.0</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E10" s="3">
+      <c r="E10" s="2">
         <v>62.0</v>
       </c>
-      <c r="F10" s="3">
+      <c r="F10" s="2">
         <v>1.0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="B11" s="3">
+        <v>106</v>
+      </c>
+      <c r="B11" s="2">
         <v>1997.0</v>
       </c>
-      <c r="C11" s="3">
+      <c r="C11" s="2">
         <v>4.0</v>
       </c>
-      <c r="D11" s="3">
+      <c r="D11" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E11" s="3">
+      <c r="E11" s="2">
         <v>48.0</v>
       </c>
-      <c r="F11" s="3">
+      <c r="F11" s="2">
         <v>1.0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="B12" s="3">
+        <v>107</v>
+      </c>
+      <c r="B12" s="2">
         <v>2008.0</v>
       </c>
-      <c r="C12" s="3">
+      <c r="C12" s="2">
         <v>4.0</v>
       </c>
-      <c r="D12" s="3">
+      <c r="D12" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E12" s="3">
+      <c r="E12" s="2">
         <v>3.0</v>
       </c>
-      <c r="F12" s="3">
+      <c r="F12" s="2">
         <v>1.0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="B13" s="3">
+        <v>108</v>
+      </c>
+      <c r="B13" s="2">
         <v>1988.0</v>
       </c>
-      <c r="C13" s="3">
+      <c r="C13" s="2">
         <v>2.0</v>
       </c>
-      <c r="D13" s="3">
+      <c r="D13" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E13" s="3">
+      <c r="E13" s="2">
         <v>18.0</v>
       </c>
-      <c r="F13" s="3">
+      <c r="F13" s="2">
         <v>1.0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="B14" s="3">
+        <v>109</v>
+      </c>
+      <c r="B14" s="2">
         <v>1996.0</v>
       </c>
-      <c r="C14" s="3">
+      <c r="C14" s="2">
         <v>2.0</v>
       </c>
-      <c r="D14" s="3">
+      <c r="D14" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E14" s="3">
+      <c r="E14" s="2">
         <v>55.0</v>
       </c>
-      <c r="F14" s="3">
+      <c r="F14" s="2">
         <v>1.0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="B15" s="3">
-        <v>2008.0</v>
-      </c>
-      <c r="C15" s="3">
+        <v>110</v>
+      </c>
+      <c r="B15" s="2">
+        <v>1996.0</v>
+      </c>
+      <c r="C15" s="2">
         <v>2.0</v>
       </c>
-      <c r="D15" s="3">
+      <c r="D15" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E15" s="3">
+      <c r="E15" s="2">
         <v>2.0</v>
       </c>
-      <c r="F15" s="3">
+      <c r="F15" s="2">
         <v>1.0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="B16" s="3">
-        <v>2008.0</v>
-      </c>
-      <c r="C16" s="3">
+        <v>111</v>
+      </c>
+      <c r="B16" s="6">
+        <v>2001.0</v>
+      </c>
+      <c r="C16" s="2">
         <v>2.0</v>
       </c>
-      <c r="D16" s="3">
+      <c r="D16" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E16" s="3">
+      <c r="E16" s="2">
         <v>1.0</v>
       </c>
-      <c r="F16" s="3">
+      <c r="F16" s="2">
         <v>1.0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="B17" s="3">
+        <v>112</v>
+      </c>
+      <c r="B17" s="2">
         <v>1993.0</v>
       </c>
-      <c r="C17" s="3">
+      <c r="C17" s="2">
         <v>3.0</v>
       </c>
-      <c r="D17" s="3">
+      <c r="D17" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E17" s="3">
+      <c r="E17" s="2">
         <v>120.0</v>
       </c>
-      <c r="F17" s="3">
+      <c r="F17" s="2">
         <v>1.0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="B18" s="3">
+        <v>113</v>
+      </c>
+      <c r="B18" s="2">
         <v>1995.0</v>
       </c>
-      <c r="C18" s="3">
+      <c r="C18" s="2">
         <v>3.0</v>
       </c>
-      <c r="D18" s="3">
+      <c r="D18" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E18" s="3">
+      <c r="E18" s="2">
         <v>88.0</v>
       </c>
-      <c r="F18" s="3">
+      <c r="F18" s="2">
         <v>1.0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="B19" s="3">
+        <v>114</v>
+      </c>
+      <c r="B19" s="2">
         <v>1997.0</v>
       </c>
-      <c r="C19" s="3">
+      <c r="C19" s="2">
         <v>3.0</v>
       </c>
-      <c r="D19" s="3">
+      <c r="D19" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E19" s="3">
+      <c r="E19" s="2">
         <v>74.0</v>
       </c>
-      <c r="F19" s="3">
+      <c r="F19" s="2">
         <v>1.0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="B20" s="3">
+        <v>115</v>
+      </c>
+      <c r="B20" s="2">
         <v>2004.0</v>
       </c>
-      <c r="C20" s="3">
+      <c r="C20" s="2">
         <v>3.0</v>
       </c>
-      <c r="D20" s="3">
+      <c r="D20" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E20" s="3">
+      <c r="E20" s="2">
         <v>30.0</v>
       </c>
-      <c r="F20" s="3">
+      <c r="F20" s="2">
         <v>1.0</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="B21" s="3">
+        <v>116</v>
+      </c>
+      <c r="B21" s="2">
         <v>2004.0</v>
       </c>
-      <c r="C21" s="3">
+      <c r="C21" s="2">
         <v>3.0</v>
       </c>
-      <c r="D21" s="3">
+      <c r="D21" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E21" s="3">
+      <c r="E21" s="2">
         <v>26.0</v>
       </c>
-      <c r="F21" s="3">
+      <c r="F21" s="2">
         <v>1.0</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="B22" s="3">
+        <v>117</v>
+      </c>
+      <c r="B22" s="2">
         <v>2005.0</v>
       </c>
-      <c r="C22" s="3">
+      <c r="C22" s="2">
         <v>3.0</v>
       </c>
-      <c r="D22" s="3">
+      <c r="D22" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E22" s="3">
+      <c r="E22" s="2">
         <v>12.0</v>
       </c>
-      <c r="F22" s="3">
+      <c r="F22" s="2">
         <v>1.0</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="B23" s="3">
+        <v>118</v>
+      </c>
+      <c r="B23" s="2">
         <v>2005.0</v>
       </c>
-      <c r="C23" s="3">
+      <c r="C23" s="2">
         <v>3.0</v>
       </c>
-      <c r="D23" s="3">
+      <c r="D23" s="2">
         <v>2026.0</v>
       </c>
-      <c r="E23" s="3">
+      <c r="E23" s="2">
         <v>9.0</v>
       </c>
-      <c r="F23" s="3">
+      <c r="F23" s="2">
         <v>1.0</v>
       </c>
     </row>
@@ -7150,19 +7165,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="7" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -8170,223 +8185,223 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B1" s="2" t="s">
+      <c r="A1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>5</v>
+      <c r="F1" s="3" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3">
+      <c r="A2" s="2">
         <v>2026.0</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="2">
         <v>1.0</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="2">
         <v>8.0</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="2">
         <v>2486.0</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2" s="2">
         <v>1.0</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>50</v>
+      <c r="F2" s="2" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3">
+      <c r="A3" s="2">
         <v>2026.0</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="2">
         <v>2.0</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="2">
         <v>5.0</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="2">
         <v>2471.0</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E3" s="2">
         <v>0.0</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>33</v>
+      <c r="F3" s="2" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3">
+      <c r="A4" s="2">
         <v>2026.0</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="2">
         <v>3.0</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="2">
         <v>4.0</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="2">
         <v>2419.5</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="2">
         <v>0.0</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>27</v>
+      <c r="F4" s="2" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3">
+      <c r="A5" s="2">
         <v>2026.0</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="2">
         <v>4.0</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="2">
         <v>9.0</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="2">
         <v>2433.0</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5" s="2">
         <v>0.0</v>
       </c>
-      <c r="F5" s="3" t="s">
-        <v>55</v>
+      <c r="F5" s="2" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3">
+      <c r="A6" s="2">
         <v>2026.0</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="2">
         <v>5.0</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="2">
         <v>7.0</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="2">
         <v>2392.5</v>
       </c>
-      <c r="E6" s="3">
+      <c r="E6" s="2">
         <v>0.0</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>44</v>
+      <c r="F6" s="2" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3">
+      <c r="A7" s="2">
         <v>2026.0</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7" s="2">
         <v>6.0</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="2">
         <v>3.0</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="2">
         <v>2480.0</v>
       </c>
-      <c r="E7" s="3">
+      <c r="E7" s="2">
         <v>0.0</v>
       </c>
-      <c r="F7" s="3" t="s">
-        <v>17</v>
+      <c r="F7" s="2" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3">
+      <c r="A8" s="2">
         <v>2026.0</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B8" s="2">
         <v>7.0</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="2">
         <v>1.0</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8" s="2">
         <v>2384.0</v>
       </c>
-      <c r="E8" s="3">
+      <c r="E8" s="2">
         <v>0.0</v>
       </c>
-      <c r="F8" s="3" t="s">
-        <v>8</v>
+      <c r="F8" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3">
+      <c r="A9" s="2">
         <v>2026.0</v>
       </c>
-      <c r="B9" s="3">
+      <c r="B9" s="2">
         <v>8.0</v>
       </c>
-      <c r="C9" s="3">
+      <c r="C9" s="2">
         <v>10.0</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="2">
         <v>2396.0</v>
       </c>
-      <c r="E9" s="3">
+      <c r="E9" s="2">
         <v>0.0</v>
       </c>
-      <c r="F9" s="3" t="s">
-        <v>61</v>
+      <c r="F9" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3">
+      <c r="A10" s="2">
         <v>2026.0</v>
       </c>
-      <c r="B10" s="3">
+      <c r="B10" s="2">
         <v>9.0</v>
       </c>
-      <c r="C10" s="3">
+      <c r="C10" s="2">
         <v>2.0</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10" s="2">
         <v>2400.0</v>
       </c>
-      <c r="E10" s="3">
+      <c r="E10" s="2">
         <v>0.0</v>
       </c>
-      <c r="F10" s="3" t="s">
-        <v>11</v>
+      <c r="F10" s="2" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3">
+      <c r="A11" s="2">
         <v>2026.0</v>
       </c>
-      <c r="B11" s="3">
+      <c r="B11" s="2">
         <v>10.0</v>
       </c>
-      <c r="C11" s="3">
+      <c r="C11" s="2">
         <v>6.0</v>
       </c>
-      <c r="D11" s="3">
+      <c r="D11" s="2">
         <v>2395.5</v>
       </c>
-      <c r="E11" s="3">
+      <c r="E11" s="2">
         <v>0.0</v>
       </c>
-      <c r="F11" s="3" t="s">
-        <v>38</v>
+      <c r="F11" s="2" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -9392,45 +9407,45 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B1" s="2" t="s">
+      <c r="A1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>5</v>
+      <c r="D1" s="3" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3">
+      <c r="A2" s="2">
         <v>2026.0</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="2">
         <v>1.0</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="2">
         <v>4.0</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>27</v>
+      <c r="D2" s="2" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3">
+      <c r="A3" s="2">
         <v>2026.0</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="2">
         <v>2.0</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="2">
         <v>8.0</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>50</v>
+      <c r="D3" s="2" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -10435,157 +10450,157 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="B1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>29</v>
+      <c r="D1" s="3" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3">
+      <c r="A2" s="2">
         <v>1.0</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="2">
         <v>2026.0</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="2">
         <v>32.0</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>7</v>
+      <c r="D2" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3">
+      <c r="A3" s="2">
         <v>2.0</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="2">
         <v>2026.0</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="2">
         <v>13.0</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>10</v>
+      <c r="D3" s="2" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3">
+      <c r="A4" s="2">
         <v>3.0</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="2">
         <v>2026.0</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="2">
         <v>34.0</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>15</v>
+      <c r="D4" s="2" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3">
+      <c r="A5" s="2">
         <v>4.0</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="2">
         <v>2026.0</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="2">
         <v>10.0</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>23</v>
+      <c r="D5" s="2" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3">
+      <c r="A6" s="2">
         <v>5.0</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="2">
         <v>2026.0</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="2">
         <v>1.0</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>32</v>
+      <c r="D6" s="2" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3">
+      <c r="A7" s="2">
         <v>6.0</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7" s="2">
         <v>2026.0</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="2">
         <v>4.0</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>36</v>
+      <c r="D7" s="2" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3">
+      <c r="A8" s="2">
         <v>7.0</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B8" s="2">
         <v>2026.0</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="2">
         <v>33.0</v>
       </c>
-      <c r="D8" s="3" t="s">
-        <v>43</v>
+      <c r="D8" s="2" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3">
+      <c r="A9" s="2">
         <v>8.0</v>
       </c>
-      <c r="B9" s="3">
+      <c r="B9" s="2">
         <v>2026.0</v>
       </c>
-      <c r="C9" s="3">
+      <c r="C9" s="2">
         <v>13.0</v>
       </c>
-      <c r="D9" s="3" t="s">
-        <v>49</v>
+      <c r="D9" s="2" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3">
+      <c r="A10" s="2">
         <v>9.0</v>
       </c>
-      <c r="B10" s="3">
+      <c r="B10" s="2">
         <v>2026.0</v>
       </c>
-      <c r="C10" s="3">
+      <c r="C10" s="2">
         <v>14.0</v>
       </c>
-      <c r="D10" s="3" t="s">
-        <v>53</v>
+      <c r="D10" s="2" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3">
+      <c r="A11" s="2">
         <v>10.0</v>
       </c>
-      <c r="B11" s="3">
+      <c r="B11" s="2">
         <v>2026.0</v>
       </c>
-      <c r="C11" s="3">
+      <c r="C11" s="2">
         <v>27.0</v>
       </c>
-      <c r="D11" s="3" t="s">
-        <v>59</v>
+      <c r="D11" s="2" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -11593,255 +11608,255 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B1" s="2" t="s">
+      <c r="A1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" s="2" t="s">
+      <c r="C1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="G1" s="2" t="s">
-        <v>127</v>
+      <c r="G1" s="3" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3">
+      <c r="A2" s="2">
         <v>2026.0</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="2">
         <v>1.0</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="3">
+      <c r="C2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" s="2">
         <v>-5.0</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2" s="2">
         <v>0.0</v>
       </c>
-      <c r="F2" s="3">
+      <c r="F2" s="2">
         <v>0.0</v>
       </c>
-      <c r="G2" s="3">
+      <c r="G2" s="2">
         <v>1027.0</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3">
+      <c r="A3" s="2">
         <v>2026.0</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="2">
         <v>2.0</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="3">
+      <c r="C3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" s="2">
         <v>-15.0</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E3" s="2">
         <v>0.0</v>
       </c>
-      <c r="F3" s="3">
+      <c r="F3" s="2">
         <v>0.0</v>
       </c>
-      <c r="G3" s="3">
+      <c r="G3" s="2">
         <v>998.0</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3">
+      <c r="A4" s="2">
         <v>2026.0</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="2">
         <v>3.0</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="3">
+      <c r="C4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" s="2">
         <v>0.0</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="2">
         <v>0.0</v>
       </c>
-      <c r="F4" s="3">
+      <c r="F4" s="2">
         <v>0.0</v>
       </c>
-      <c r="G4" s="3">
+      <c r="G4" s="2">
         <v>1034.0</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3">
+      <c r="A5" s="2">
         <v>2026.0</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="2">
         <v>4.0</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="D5" s="3">
+      <c r="C5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" s="2">
         <v>10.0</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5" s="2">
         <v>10.0</v>
       </c>
-      <c r="F5" s="3">
+      <c r="F5" s="2">
         <v>0.0</v>
       </c>
-      <c r="G5" s="3">
+      <c r="G5" s="2">
         <v>1030.0</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3">
+      <c r="A6" s="2">
         <v>2026.0</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="2">
         <v>5.0</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="D6" s="3">
+      <c r="C6" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D6" s="2">
         <v>15.0</v>
       </c>
-      <c r="E6" s="3">
+      <c r="E6" s="2">
         <v>0.0</v>
       </c>
-      <c r="F6" s="3">
+      <c r="F6" s="2">
         <v>0.0</v>
       </c>
-      <c r="G6" s="3">
+      <c r="G6" s="2">
         <v>1016.0</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3">
+      <c r="A7" s="2">
         <v>2026.0</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7" s="2">
         <v>6.0</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="D7" s="3">
+      <c r="C7" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D7" s="2">
         <v>-20.0</v>
       </c>
-      <c r="E7" s="3">
+      <c r="E7" s="2">
         <v>0.0</v>
       </c>
-      <c r="F7" s="3">
+      <c r="F7" s="2">
         <v>0.0</v>
       </c>
-      <c r="G7" s="3">
+      <c r="G7" s="2">
         <v>984.0</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3">
+      <c r="A8" s="2">
         <v>2026.0</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B8" s="2">
         <v>7.0</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D8" s="3">
+      <c r="C8" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D8" s="2">
         <v>0.0</v>
       </c>
-      <c r="E8" s="3">
+      <c r="E8" s="2">
         <v>0.0</v>
       </c>
-      <c r="F8" s="3">
+      <c r="F8" s="2">
         <v>0.0</v>
       </c>
-      <c r="G8" s="3">
+      <c r="G8" s="2">
         <v>1033.0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3">
+      <c r="A9" s="2">
         <v>2026.0</v>
       </c>
-      <c r="B9" s="3">
+      <c r="B9" s="2">
         <v>8.0</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="D9" s="3">
+      <c r="C9" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D9" s="2">
         <v>25.0</v>
       </c>
-      <c r="E9" s="3">
+      <c r="E9" s="2">
         <v>0.0</v>
       </c>
-      <c r="F9" s="3">
+      <c r="F9" s="2">
         <v>10.0</v>
       </c>
-      <c r="G9" s="3">
+      <c r="G9" s="2">
         <v>1048.0</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3">
+      <c r="A10" s="2">
         <v>2026.0</v>
       </c>
-      <c r="B10" s="3">
+      <c r="B10" s="2">
         <v>9.0</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="D10" s="3">
+      <c r="C10" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D10" s="2">
         <v>5.0</v>
       </c>
-      <c r="E10" s="3">
+      <c r="E10" s="2">
         <v>0.0</v>
       </c>
-      <c r="F10" s="3">
+      <c r="F10" s="2">
         <v>0.0</v>
       </c>
-      <c r="G10" s="3">
+      <c r="G10" s="2">
         <v>1019.0</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3">
+      <c r="A11" s="2">
         <v>2026.0</v>
       </c>
-      <c r="B11" s="3">
+      <c r="B11" s="2">
         <v>10.0</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="D11" s="3">
+      <c r="C11" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D11" s="2">
         <v>-10.0</v>
       </c>
-      <c r="E11" s="3">
+      <c r="E11" s="2">
         <v>0.0</v>
       </c>
-      <c r="F11" s="3">
+      <c r="F11" s="2">
         <v>0.0</v>
       </c>
-      <c r="G11" s="3">
+      <c r="G11" s="2">
         <v>1017.0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Riconferme 2026: 46 contratti dalle rose 25-26
Inserite in Gestione.xlsx le riconferme di tutte e 10 le squadre
(AnnoInizio 2026, scadenza 2029) e rimosse le righe demo.

Versiona anche le rose e i riscatti 25-26 in CSV; gli screenshot PNG
della stessa cartella restano fuori da Git (decine di MB su un repo
pubblico).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dati/Gestione.xlsx
+++ b/dati/Gestione.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="170">
   <si>
     <t>FANTA BRECCIA — foglio di gestione</t>
   </si>
@@ -33,61 +33,130 @@
     <t>ID</t>
   </si>
   <si>
+    <t>Giocatore</t>
+  </si>
+  <si>
+    <t>Allenatore</t>
+  </si>
+  <si>
+    <t>Squadra</t>
+  </si>
+  <si>
     <t>Questo file e' la fonte unica dei dati del sito.</t>
   </si>
   <si>
+    <t>Mindo</t>
+  </si>
+  <si>
+    <t>Chentus</t>
+  </si>
+  <si>
     <t>Dopo averlo modificato e SALVATO: doppio click su aggiorna.bat</t>
   </si>
   <si>
+    <t>Alessio Cocchieri &amp; Febio</t>
+  </si>
+  <si>
+    <t>Anno</t>
+  </si>
+  <si>
+    <t>MALLOREDDUS FC</t>
+  </si>
+  <si>
     <t>Foglio</t>
   </si>
   <si>
-    <t>Allenatore</t>
-  </si>
-  <si>
-    <t>Anno</t>
-  </si>
-  <si>
-    <t>Squadra</t>
+    <t>PietroPJ</t>
+  </si>
+  <si>
+    <t>Sporting Garra</t>
   </si>
   <si>
     <t>Nome</t>
   </si>
   <si>
-    <t>Giocatore</t>
+    <t>Max Allegri</t>
+  </si>
+  <si>
+    <t>Whiteam FC</t>
+  </si>
+  <si>
+    <t>AnnoNascita</t>
+  </si>
+  <si>
+    <t>Fil e Pacciansss &amp; sono innocenti</t>
+  </si>
+  <si>
+    <t>TurettaEPacciani FC</t>
   </si>
   <si>
     <t>Tabella SQLite</t>
   </si>
   <si>
+    <t>Alessio Bruni</t>
+  </si>
+  <si>
+    <t>IDSquadra</t>
+  </si>
+  <si>
+    <t>Nkunku Settete</t>
+  </si>
+  <si>
     <t>Contenuto</t>
   </si>
   <si>
+    <t>AnnoInizio</t>
+  </si>
+  <si>
+    <t>deiu &amp; Bep</t>
+  </si>
+  <si>
+    <t>Mapi Group</t>
+  </si>
+  <si>
+    <t>PrezzoAcquisto</t>
+  </si>
+  <si>
     <t>AnagraficaSquadre</t>
   </si>
   <si>
     <t>teams</t>
   </si>
   <si>
-    <t>Mindo</t>
+    <t>Attivo</t>
+  </si>
+  <si>
+    <t>CariBam &amp; sickroul</t>
   </si>
   <si>
     <t>Squadre e allenatori (qui stanno gli ID)</t>
   </si>
   <si>
-    <t>Chentus</t>
+    <t>Roul e il socio</t>
+  </si>
+  <si>
+    <t>Luca baffi e tabacchi</t>
+  </si>
+  <si>
+    <t>Davis K.</t>
   </si>
   <si>
     <t>CambioNome</t>
   </si>
   <si>
+    <t>Compagnia Ascolana Sigari</t>
+  </si>
+  <si>
     <t>cambio_nome</t>
   </si>
   <si>
     <t>Nome della squadra per anno</t>
   </si>
   <si>
-    <t>Alessio Cocchieri &amp; Febio</t>
+    <t>mister zeman</t>
+  </si>
+  <si>
+    <t>Tridente demoniaco</t>
   </si>
   <si>
     <t>Contratti</t>
@@ -96,138 +165,96 @@
     <t>contracts + players</t>
   </si>
   <si>
-    <t>MALLOREDDUS FC</t>
-  </si>
-  <si>
     <t>Contratti di riconferma</t>
   </si>
   <si>
+    <t>Thorstvedt</t>
+  </si>
+  <si>
     <t>Svincoli</t>
   </si>
   <si>
-    <t>PietroPJ</t>
-  </si>
-  <si>
     <t>contract_releases</t>
   </si>
   <si>
-    <t>AnnoNascita</t>
-  </si>
-  <si>
-    <t>Sporting Garra</t>
-  </si>
-  <si>
     <t>Svincoli: storico e penali</t>
   </si>
   <si>
-    <t>IDSquadra</t>
-  </si>
-  <si>
     <t>Classifiche</t>
   </si>
   <si>
-    <t>AnnoInizio</t>
-  </si>
-  <si>
-    <t>Max Allegri</t>
-  </si>
-  <si>
     <t>season_rankings</t>
   </si>
   <si>
-    <t>Whiteam FC</t>
-  </si>
-  <si>
     <t>Classifica di campionato</t>
   </si>
   <si>
+    <t>Da Cunha</t>
+  </si>
+  <si>
     <t>Coppa</t>
   </si>
   <si>
-    <t>Fil e Pacciansss &amp; sono innocenti</t>
-  </si>
-  <si>
     <t>coppa</t>
   </si>
   <si>
-    <t>TurettaEPacciani FC</t>
-  </si>
-  <si>
     <t>Podio della coppa</t>
   </si>
   <si>
     <t>CreditiAsta</t>
   </si>
   <si>
+    <t>Samardzic</t>
+  </si>
+  <si>
     <t>credit_residual</t>
   </si>
   <si>
-    <t>Alessio Bruni</t>
-  </si>
-  <si>
     <t>Crediti avanzati a fine stagione</t>
   </si>
   <si>
-    <t>Nkunku Settete</t>
-  </si>
-  <si>
     <t>CreditiAnnoNuovo</t>
   </si>
   <si>
-    <t>PrezzoAcquisto</t>
-  </si>
-  <si>
     <t>crediti_anno_nuovo</t>
   </si>
   <si>
-    <t>deiu &amp; Bep</t>
-  </si>
-  <si>
     <t>Budget della stagione nuova</t>
   </si>
   <si>
-    <t>Attivo</t>
-  </si>
-  <si>
-    <t>Mapi Group</t>
+    <t>Ghilardi</t>
   </si>
   <si>
     <t>FOGLIO CONTRATTI</t>
   </si>
   <si>
-    <t>CariBam &amp; sickroul</t>
-  </si>
-  <si>
     <t>nome del calciatore, scritto per esteso</t>
   </si>
   <si>
-    <t>Alvarez</t>
-  </si>
-  <si>
-    <t>Roul e il socio</t>
+    <t>Vlasic</t>
   </si>
   <si>
     <t>solo l'anno: da qui dipende la categoria A/B/C</t>
   </si>
   <si>
-    <t>Luca baffi e tabacchi</t>
-  </si>
-  <si>
     <t>ID come in AnagraficaSquadre</t>
   </si>
   <si>
-    <t>Compagnia Ascolana Sigari</t>
+    <t>Lauriente</t>
   </si>
   <si>
     <t>anno della riconferma</t>
   </si>
   <si>
-    <t>mister zeman</t>
+    <t>Bisseck</t>
   </si>
   <si>
     <t>prezzo pagato all'asta: non cambia mai</t>
   </si>
   <si>
+    <t>Rowe</t>
+  </si>
+  <si>
     <t>1 se in corso, 0 se chiuso</t>
   </si>
   <si>
@@ -237,18 +264,18 @@
     <t>e' sempre AnnoInizio + 3 (regolamento par. 1)</t>
   </si>
   <si>
-    <t>Perin</t>
+    <t>Rodriguez Je.</t>
   </si>
   <si>
     <t>FOGLIO SVINCOLI</t>
   </si>
   <si>
-    <t>Tridente demoniaco</t>
-  </si>
-  <si>
     <t>stesso nome scritto in Contratti</t>
   </si>
   <si>
+    <t>Bernasconi</t>
+  </si>
+  <si>
     <t>la squadra che lo svincola</t>
   </si>
   <si>
@@ -258,15 +285,18 @@
     <t>anno in cui viene svincolato</t>
   </si>
   <si>
+    <t>Ramon</t>
+  </si>
+  <si>
     <t>Penale</t>
   </si>
   <si>
-    <t>Conti</t>
-  </si>
-  <si>
     <t>LASCIALA VUOTA: la calcola il sistema.</t>
   </si>
   <si>
+    <t>Dimarco</t>
+  </si>
+  <si>
     <t>Compilala solo per forzare un valore diverso.</t>
   </si>
   <si>
@@ -276,13 +306,16 @@
     <t>motivo, facoltativo</t>
   </si>
   <si>
+    <t>Gaetano</t>
+  </si>
+  <si>
     <t>QUANDO SVINCOLI UN GIOCATORE</t>
   </si>
   <si>
     <t>1. Aggiungi la riga qui in Svincoli</t>
   </si>
   <si>
-    <t>Donati</t>
+    <t>Malen</t>
   </si>
   <si>
     <t>2. Metti Attivo = 0 nella sua riga di Contratti</t>
@@ -294,6 +327,9 @@
     <t>CATEGORIE (sull'anno di riferimento)</t>
   </si>
   <si>
+    <t>Douvikas</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
@@ -303,12 +339,12 @@
     <t>illimitati</t>
   </si>
   <si>
+    <t>Frattesi</t>
+  </si>
+  <si>
     <t>B</t>
   </si>
   <si>
-    <t>Ferraro</t>
-  </si>
-  <si>
     <t>eta' &lt;= 25</t>
   </si>
   <si>
@@ -321,13 +357,16 @@
     <t>oltre i 25</t>
   </si>
   <si>
+    <t>Martinez Jo.</t>
+  </si>
+  <si>
     <t>massimo 3</t>
   </si>
   <si>
     <t>CREDITI DELLA STAGIONE NUOVA</t>
   </si>
   <si>
-    <t>Gatti</t>
+    <t>Bonny</t>
   </si>
   <si>
     <t>Non si compilano a mano.</t>
@@ -336,52 +375,85 @@
     <t>strumenti\calcola_crediti.py li calcola</t>
   </si>
   <si>
-    <t>Moretti</t>
-  </si>
-  <si>
-    <t>Rinaldi</t>
-  </si>
-  <si>
-    <t>Santoro</t>
-  </si>
-  <si>
-    <t>Lombardi</t>
-  </si>
-  <si>
-    <t>Ricci</t>
-  </si>
-  <si>
-    <t>Marino</t>
-  </si>
-  <si>
-    <t>Baggio</t>
-  </si>
-  <si>
-    <t>Greco</t>
-  </si>
-  <si>
-    <t>Romano</t>
-  </si>
-  <si>
-    <t>Martini</t>
-  </si>
-  <si>
-    <t>Costa</t>
-  </si>
-  <si>
-    <t>Serra</t>
-  </si>
-  <si>
-    <t>Pellegrini</t>
-  </si>
-  <si>
-    <t>Vitale</t>
+    <t>Atta</t>
+  </si>
+  <si>
+    <t>Esposito F.P.</t>
+  </si>
+  <si>
+    <t>Okoye</t>
+  </si>
+  <si>
+    <t>Kalulu</t>
+  </si>
+  <si>
+    <t>Solet</t>
+  </si>
+  <si>
+    <t>Belghali</t>
+  </si>
+  <si>
+    <t>Baturina</t>
+  </si>
+  <si>
+    <t>McKennie</t>
+  </si>
+  <si>
+    <t>Butez</t>
+  </si>
+  <si>
+    <t>Muric</t>
+  </si>
+  <si>
+    <t>Gila</t>
+  </si>
+  <si>
+    <t>Cambiaghi</t>
+  </si>
+  <si>
+    <t>Fazzini</t>
+  </si>
+  <si>
+    <t>Lucumi</t>
+  </si>
+  <si>
+    <t>Ostigard</t>
+  </si>
+  <si>
+    <t>Zaniolo</t>
+  </si>
+  <si>
+    <t>Diao</t>
+  </si>
+  <si>
+    <t>Carnesecchi</t>
+  </si>
+  <si>
+    <t>Wesley</t>
+  </si>
+  <si>
+    <t>Rrahmani</t>
+  </si>
+  <si>
+    <t>Valle</t>
   </si>
   <si>
     <t>Colombo</t>
   </si>
   <si>
-    <t>Esposito</t>
+    <t>Simeone</t>
+  </si>
+  <si>
+    <t>Mancini</t>
+  </si>
+  <si>
+    <t>Casadei</t>
+  </si>
+  <si>
+    <t>Pierotti</t>
+  </si>
+  <si>
+    <t>Dovbyk</t>
   </si>
   <si>
     <t>Posizione</t>
@@ -469,21 +541,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <sz val="11.0"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14.0"/>
-      <color rgb="FF7A3E12"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
@@ -493,13 +553,31 @@
       <sz val="11.0"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14.0"/>
+      <color rgb="FF7A3E12"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11.0"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="6">
@@ -546,26 +624,32 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="1" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="right" vertical="bottom"/>
+    </xf>
+    <xf borderId="1" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="5" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -824,303 +908,303 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="2" t="s">
+      <c r="C17" s="3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="s">
+      <c r="C18" s="3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>67</v>
+      <c r="C22" s="3" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>69</v>
+      <c r="A23" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1"/>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="4" t="s">
-        <v>71</v>
+      <c r="A25" s="5" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>73</v>
+      <c r="A26" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>74</v>
+      <c r="A27" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>76</v>
+      <c r="A28" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>79</v>
+      <c r="A29" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="C30" s="2" t="s">
-        <v>80</v>
+      <c r="C30" s="3" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>82</v>
+      <c r="A31" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1"/>
     <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="4" t="s">
-        <v>83</v>
+      <c r="A33" s="5" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="2" t="s">
-        <v>84</v>
+      <c r="A34" s="3" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
-      <c r="A35" s="2" t="s">
-        <v>86</v>
+      <c r="A35" s="3" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
-      <c r="A36" s="2" t="s">
-        <v>87</v>
+      <c r="A36" s="3" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1"/>
     <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="4" t="s">
-        <v>88</v>
+      <c r="A38" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
-      <c r="A39" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>91</v>
+      <c r="A39" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
-      <c r="A40" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>95</v>
+      <c r="A40" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
-      <c r="A41" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>98</v>
+      <c r="A41" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1"/>
     <row r="43" ht="15.75" customHeight="1">
-      <c r="A43" s="4" t="s">
-        <v>99</v>
+      <c r="A43" s="5" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
-      <c r="A44" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>102</v>
+      <c r="A44" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1"/>
@@ -2104,342 +2188,342 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>128</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>129</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>130</v>
+      <c r="A1" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="C2" s="2">
+      <c r="A2" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="C2" s="3">
         <v>1000.0</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="3">
         <v>2999.0</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>132</v>
+      <c r="F2" s="3" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="C3" s="2">
+      <c r="A3" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="C3" s="3">
         <v>950.0</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="3">
         <v>2999.0</v>
       </c>
-      <c r="F3" s="2" t="s">
-        <v>134</v>
+      <c r="F3" s="3" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="C4" s="2">
+      <c r="A4" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="C4" s="3">
         <v>1100.0</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="3">
         <v>2999.0</v>
       </c>
-      <c r="F4" s="2" t="s">
-        <v>136</v>
+      <c r="F4" s="3" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="C5" s="2">
+      <c r="A5" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="C5" s="3">
         <v>900.0</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="3">
         <v>2999.0</v>
       </c>
-      <c r="F5" s="2" t="s">
-        <v>138</v>
+      <c r="F5" s="3" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="B6" s="2">
+      <c r="A6" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="B6" s="3">
         <v>1.0</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="3">
         <v>25.0</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="3">
         <v>2999.0</v>
       </c>
-      <c r="F6" s="2" t="s">
-        <v>140</v>
+      <c r="F6" s="3" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="B7" s="2">
+      <c r="A7" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="B7" s="3">
         <v>2.0</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="3">
         <v>15.0</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="3">
         <v>2999.0</v>
       </c>
-      <c r="F7" s="2" t="s">
-        <v>140</v>
+      <c r="F7" s="3" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="B8" s="2">
+      <c r="A8" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="B8" s="3">
         <v>3.0</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8" s="3">
         <v>10.0</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="3">
         <v>2999.0</v>
       </c>
-      <c r="F8" s="2" t="s">
-        <v>140</v>
+      <c r="F8" s="3" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="B9" s="2">
+      <c r="A9" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="B9" s="3">
         <v>4.0</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C9" s="3">
         <v>5.0</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="3">
         <v>2999.0</v>
       </c>
-      <c r="F9" s="2" t="s">
-        <v>140</v>
+      <c r="F9" s="3" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="B10" s="2">
+      <c r="A10" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="B10" s="3">
         <v>5.0</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" s="3">
         <v>0.0</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="3">
         <v>2999.0</v>
       </c>
-      <c r="F10" s="2" t="s">
-        <v>140</v>
+      <c r="F10" s="3" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="B11" s="2">
+      <c r="A11" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="B11" s="3">
         <v>6.0</v>
       </c>
-      <c r="C11" s="2">
+      <c r="C11" s="3">
         <v>0.0</v>
       </c>
-      <c r="D11" s="2">
+      <c r="D11" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="3">
         <v>2999.0</v>
       </c>
-      <c r="F11" s="2" t="s">
-        <v>140</v>
+      <c r="F11" s="3" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="B12" s="2">
+      <c r="A12" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="B12" s="3">
         <v>7.0</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C12" s="3">
         <v>-5.0</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="3">
         <v>2999.0</v>
       </c>
-      <c r="F12" s="2" t="s">
-        <v>140</v>
+      <c r="F12" s="3" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="B13" s="2">
+      <c r="A13" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="B13" s="3">
         <v>8.0</v>
       </c>
-      <c r="C13" s="2">
+      <c r="C13" s="3">
         <v>-10.0</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="3">
         <v>2999.0</v>
       </c>
-      <c r="F13" s="2" t="s">
-        <v>140</v>
+      <c r="F13" s="3" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="B14" s="2">
+      <c r="A14" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="B14" s="3">
         <v>9.0</v>
       </c>
-      <c r="C14" s="2">
+      <c r="C14" s="3">
         <v>-15.0</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="3">
         <v>2999.0</v>
       </c>
-      <c r="F14" s="2" t="s">
-        <v>140</v>
+      <c r="F14" s="3" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="B15" s="2">
+      <c r="A15" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="B15" s="3">
         <v>10.0</v>
       </c>
-      <c r="C15" s="2">
+      <c r="C15" s="3">
         <v>-20.0</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="3">
         <v>2999.0</v>
       </c>
-      <c r="F15" s="2" t="s">
-        <v>140</v>
+      <c r="F15" s="3" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="C16" s="2">
+      <c r="A16" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="C16" s="3">
         <v>10.0</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="3">
         <v>2999.0</v>
       </c>
-      <c r="F16" s="2" t="s">
-        <v>142</v>
+      <c r="F16" s="3" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C17" s="2">
+      <c r="A17" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C17" s="3">
         <v>10.0</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="3">
         <v>2999.0</v>
       </c>
-      <c r="F17" s="2" t="s">
-        <v>143</v>
+      <c r="F17" s="3" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="C18" s="2">
+      <c r="A18" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="C18" s="3">
         <v>50.0</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="3">
         <v>2999.0</v>
       </c>
-      <c r="F18" s="2" t="s">
-        <v>145</v>
+      <c r="F18" s="3" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -3444,124 +3528,124 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" s="3" t="s">
+      <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2">
-        <v>1.0</v>
-      </c>
-      <c r="B2" s="2" t="s">
+    <row r="3">
+      <c r="A3" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="2" t="s">
+    </row>
+    <row r="5">
+      <c r="A5" s="3">
+        <v>4.0</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2">
-        <v>2.0</v>
-      </c>
-      <c r="B3" s="2" t="s">
+      <c r="C5" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3">
+        <v>5.0</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2">
-        <v>3.0</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2">
-        <v>4.0</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C5" s="2" t="s">
+    </row>
+    <row r="7">
+      <c r="A7" s="3">
+        <v>6.0</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3">
+        <v>7.0</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3">
+        <v>8.0</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3">
+        <v>9.0</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2">
-        <v>5.0</v>
-      </c>
-      <c r="B6" s="2" t="s">
+      <c r="C10" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2">
-        <v>6.0</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2">
-        <v>7.0</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2">
-        <v>8.0</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2">
-        <v>9.0</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="11">
-      <c r="A11" s="2">
+      <c r="A11" s="3">
         <v>10.0</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>72</v>
+      <c r="B11" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -4565,124 +4649,124 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>8</v>
+      <c r="B1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2">
+      <c r="A2" s="3">
         <v>1.0</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="3">
         <v>2026.0</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>16</v>
+      <c r="C2" s="3" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2">
+      <c r="A3" s="3">
         <v>2.0</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="3">
         <v>2026.0</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>23</v>
+      <c r="C3" s="3" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2">
+      <c r="A4" s="3">
         <v>3.0</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="3">
         <v>2026.0</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>29</v>
+      <c r="C4" s="3" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2">
+      <c r="A5" s="3">
         <v>4.0</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="3">
         <v>2026.0</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>36</v>
+      <c r="C5" s="3" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2">
+      <c r="A6" s="3">
         <v>5.0</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" s="3">
         <v>2026.0</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>41</v>
+      <c r="C6" s="3" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2">
+      <c r="A7" s="3">
         <v>6.0</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7" s="3">
         <v>2026.0</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>47</v>
+      <c r="C7" s="3" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2">
+      <c r="A8" s="3">
         <v>7.0</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B8" s="3">
         <v>2026.0</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>54</v>
+      <c r="C8" s="3" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2">
+      <c r="A9" s="3">
         <v>8.0</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B9" s="3">
         <v>2026.0</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>59</v>
+      <c r="C9" s="3" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2">
+      <c r="A10" s="3">
         <v>9.0</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10" s="3">
         <v>2026.0</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>63</v>
+      <c r="C10" s="3" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2">
+      <c r="A11" s="3">
         <v>10.0</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11" s="3">
         <v>2026.0</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>72</v>
+      <c r="C11" s="3" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -5689,417 +5773,407 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>53</v>
+      <c r="A1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="B2" s="2">
-        <v>2006.0</v>
-      </c>
-      <c r="C2" s="2">
-        <v>1.0</v>
-      </c>
-      <c r="D2" s="2">
+        <v>37</v>
+      </c>
+      <c r="B2" s="6">
+        <v>1998.0</v>
+      </c>
+      <c r="C2" s="6">
+        <v>4.0</v>
+      </c>
+      <c r="D2" s="6">
         <v>2026.0</v>
       </c>
-      <c r="E2" s="2">
-        <v>21.0</v>
-      </c>
-      <c r="F2" s="2">
+      <c r="E2" s="6">
+        <v>33.0</v>
+      </c>
+      <c r="F2" s="6">
         <v>1.0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="B3" s="2">
-        <v>2006.0</v>
-      </c>
-      <c r="C3" s="2">
+        <v>47</v>
+      </c>
+      <c r="B3" s="6">
+        <v>1999.0</v>
+      </c>
+      <c r="C3" s="6">
+        <v>4.0</v>
+      </c>
+      <c r="D3" s="6">
+        <v>2026.0</v>
+      </c>
+      <c r="E3" s="6">
         <v>1.0</v>
       </c>
-      <c r="D3" s="2">
-        <v>2026.0</v>
-      </c>
-      <c r="E3" s="2">
-        <v>11.0</v>
-      </c>
-      <c r="F3" s="2">
+      <c r="F3" s="6">
         <v>1.0</v>
       </c>
-      <c r="I3" s="2">
-        <v>2003.0</v>
-      </c>
+      <c r="I3" s="3"/>
     </row>
     <row r="4">
       <c r="A4" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="B4" s="2">
-        <v>2006.0</v>
-      </c>
-      <c r="C4" s="2">
+        <v>54</v>
+      </c>
+      <c r="B4" s="6">
+        <v>2001.0</v>
+      </c>
+      <c r="C4" s="6">
+        <v>4.0</v>
+      </c>
+      <c r="D4" s="6">
+        <v>2026.0</v>
+      </c>
+      <c r="E4" s="6">
         <v>1.0</v>
       </c>
-      <c r="D4" s="2">
-        <v>2026.0</v>
-      </c>
-      <c r="E4" s="2">
-        <v>24.0</v>
-      </c>
-      <c r="F4" s="2">
+      <c r="F4" s="6">
         <v>1.0</v>
       </c>
-      <c r="I4" s="2">
-        <v>1997.0</v>
-      </c>
+      <c r="I4" s="3"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="B5" s="2">
-        <v>2006.0</v>
-      </c>
-      <c r="C5" s="2">
+        <v>59</v>
+      </c>
+      <c r="B5" s="6">
+        <v>2002.0</v>
+      </c>
+      <c r="C5" s="6">
+        <v>4.0</v>
+      </c>
+      <c r="D5" s="6">
+        <v>2026.0</v>
+      </c>
+      <c r="E5" s="6">
+        <v>14.0</v>
+      </c>
+      <c r="F5" s="6">
         <v>1.0</v>
       </c>
-      <c r="D5" s="2">
-        <v>2026.0</v>
-      </c>
-      <c r="E5" s="2">
-        <v>31.0</v>
-      </c>
-      <c r="F5" s="2">
-        <v>1.0</v>
-      </c>
-      <c r="I5" s="2">
-        <v>1996.0</v>
-      </c>
+      <c r="I5" s="3"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="B6" s="2">
-        <v>2006.0</v>
-      </c>
-      <c r="C6" s="2">
+        <v>65</v>
+      </c>
+      <c r="B6" s="6">
+        <v>2003.0</v>
+      </c>
+      <c r="C6" s="6">
+        <v>4.0</v>
+      </c>
+      <c r="D6" s="6">
+        <v>2026.0</v>
+      </c>
+      <c r="E6" s="6">
         <v>1.0</v>
       </c>
-      <c r="D6" s="2">
-        <v>2026.0</v>
-      </c>
-      <c r="E6" s="2">
-        <v>122.0</v>
-      </c>
-      <c r="F6" s="2">
+      <c r="F6" s="6">
         <v>1.0</v>
       </c>
-      <c r="I6" s="2">
-        <v>1996.0</v>
-      </c>
+      <c r="I6" s="3"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="B7" s="2">
-        <v>2006.0</v>
-      </c>
-      <c r="C7" s="2">
+        <v>68</v>
+      </c>
+      <c r="B7" s="6">
+        <v>1997.0</v>
+      </c>
+      <c r="C7" s="6">
+        <v>3.0</v>
+      </c>
+      <c r="D7" s="6">
+        <v>2026.0</v>
+      </c>
+      <c r="E7" s="6">
+        <v>41.0</v>
+      </c>
+      <c r="F7" s="6">
         <v>1.0</v>
       </c>
-      <c r="D7" s="2">
-        <v>2026.0</v>
-      </c>
-      <c r="E7" s="2">
-        <v>1.0</v>
-      </c>
-      <c r="F7" s="2">
-        <v>1.0</v>
-      </c>
-      <c r="I7" s="2">
-        <v>2001.0</v>
-      </c>
+      <c r="I7" s="3"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="B8" s="2">
-        <v>2000.0</v>
-      </c>
-      <c r="C8" s="2">
-        <v>4.0</v>
-      </c>
-      <c r="D8" s="2">
+        <v>71</v>
+      </c>
+      <c r="B8" s="6">
+        <v>1998.0</v>
+      </c>
+      <c r="C8" s="6">
+        <v>3.0</v>
+      </c>
+      <c r="D8" s="6">
         <v>2026.0</v>
       </c>
-      <c r="E8" s="2">
-        <v>210.0</v>
-      </c>
-      <c r="F8" s="2">
+      <c r="E8" s="6">
+        <v>43.0</v>
+      </c>
+      <c r="F8" s="6">
         <v>1.0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="B9" s="2">
-        <v>1997.0</v>
-      </c>
-      <c r="C9" s="2">
-        <v>4.0</v>
-      </c>
-      <c r="D9" s="2">
+        <v>73</v>
+      </c>
+      <c r="B9" s="6">
+        <v>2000.0</v>
+      </c>
+      <c r="C9" s="6">
+        <v>3.0</v>
+      </c>
+      <c r="D9" s="6">
         <v>2026.0</v>
       </c>
-      <c r="E9" s="2">
-        <v>95.0</v>
-      </c>
-      <c r="F9" s="2">
+      <c r="E9" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="F9" s="6">
         <v>1.0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="B10" s="2">
-        <v>1999.0</v>
-      </c>
-      <c r="C10" s="2">
-        <v>4.0</v>
-      </c>
-      <c r="D10" s="2">
+        <v>75</v>
+      </c>
+      <c r="B10" s="6">
+        <v>2003.0</v>
+      </c>
+      <c r="C10" s="6">
+        <v>3.0</v>
+      </c>
+      <c r="D10" s="6">
         <v>2026.0</v>
       </c>
-      <c r="E10" s="2">
-        <v>62.0</v>
-      </c>
-      <c r="F10" s="2">
+      <c r="E10" s="6">
+        <v>17.0</v>
+      </c>
+      <c r="F10" s="6">
         <v>1.0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="B11" s="2">
-        <v>1997.0</v>
-      </c>
-      <c r="C11" s="2">
-        <v>4.0</v>
-      </c>
-      <c r="D11" s="2">
+        <v>79</v>
+      </c>
+      <c r="B11" s="6">
+        <v>2005.0</v>
+      </c>
+      <c r="C11" s="6">
+        <v>3.0</v>
+      </c>
+      <c r="D11" s="6">
         <v>2026.0</v>
       </c>
-      <c r="E11" s="2">
-        <v>48.0</v>
-      </c>
-      <c r="F11" s="2">
+      <c r="E11" s="6">
+        <v>6.0</v>
+      </c>
+      <c r="F11" s="6">
         <v>1.0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="B12" s="2">
-        <v>2008.0</v>
-      </c>
-      <c r="C12" s="2">
-        <v>4.0</v>
-      </c>
-      <c r="D12" s="2">
+        <v>82</v>
+      </c>
+      <c r="B12" s="6">
+        <v>2003.0</v>
+      </c>
+      <c r="C12" s="6">
+        <v>8.0</v>
+      </c>
+      <c r="D12" s="6">
         <v>2026.0</v>
       </c>
-      <c r="E12" s="2">
-        <v>3.0</v>
-      </c>
-      <c r="F12" s="2">
+      <c r="E12" s="6">
+        <v>5.0</v>
+      </c>
+      <c r="F12" s="6">
         <v>1.0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="B13" s="2">
-        <v>1988.0</v>
-      </c>
-      <c r="C13" s="2">
-        <v>2.0</v>
-      </c>
-      <c r="D13" s="2">
+        <v>86</v>
+      </c>
+      <c r="B13" s="6">
+        <v>2005.0</v>
+      </c>
+      <c r="C13" s="6">
+        <v>8.0</v>
+      </c>
+      <c r="D13" s="6">
         <v>2026.0</v>
       </c>
-      <c r="E13" s="2">
-        <v>18.0</v>
-      </c>
-      <c r="F13" s="2">
+      <c r="E13" s="6">
+        <v>10.0</v>
+      </c>
+      <c r="F13" s="6">
         <v>1.0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="B14" s="2">
-        <v>1996.0</v>
-      </c>
-      <c r="C14" s="2">
-        <v>2.0</v>
-      </c>
-      <c r="D14" s="2">
+        <v>89</v>
+      </c>
+      <c r="B14" s="6">
+        <v>1997.0</v>
+      </c>
+      <c r="C14" s="6">
+        <v>8.0</v>
+      </c>
+      <c r="D14" s="6">
         <v>2026.0</v>
       </c>
-      <c r="E14" s="2">
-        <v>55.0</v>
-      </c>
-      <c r="F14" s="2">
+      <c r="E14" s="6">
+        <v>73.0</v>
+      </c>
+      <c r="F14" s="6">
         <v>1.0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="B15" s="2">
-        <v>1996.0</v>
-      </c>
-      <c r="C15" s="2">
-        <v>2.0</v>
-      </c>
-      <c r="D15" s="2">
+        <v>93</v>
+      </c>
+      <c r="B15" s="6">
+        <v>2000.0</v>
+      </c>
+      <c r="C15" s="6">
+        <v>8.0</v>
+      </c>
+      <c r="D15" s="6">
         <v>2026.0</v>
       </c>
-      <c r="E15" s="2">
-        <v>2.0</v>
-      </c>
-      <c r="F15" s="2">
+      <c r="E15" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="F15" s="6">
         <v>1.0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="s">
-        <v>111</v>
+        <v>96</v>
       </c>
       <c r="B16" s="6">
-        <v>2001.0</v>
-      </c>
-      <c r="C16" s="2">
-        <v>2.0</v>
-      </c>
-      <c r="D16" s="2">
+        <v>1999.0</v>
+      </c>
+      <c r="C16" s="6">
+        <v>8.0</v>
+      </c>
+      <c r="D16" s="6">
         <v>2026.0</v>
       </c>
-      <c r="E16" s="2">
-        <v>1.0</v>
-      </c>
-      <c r="F16" s="2">
+      <c r="E16" s="6">
+        <v>210.0</v>
+      </c>
+      <c r="F16" s="6">
         <v>1.0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="B17" s="2">
-        <v>1993.0</v>
-      </c>
-      <c r="C17" s="2">
-        <v>3.0</v>
-      </c>
-      <c r="D17" s="2">
+        <v>100</v>
+      </c>
+      <c r="B17" s="6">
+        <v>1999.0</v>
+      </c>
+      <c r="C17" s="6">
+        <v>9.0</v>
+      </c>
+      <c r="D17" s="6">
         <v>2026.0</v>
       </c>
-      <c r="E17" s="2">
-        <v>120.0</v>
-      </c>
-      <c r="F17" s="2">
+      <c r="E17" s="6">
+        <v>24.0</v>
+      </c>
+      <c r="F17" s="6">
         <v>1.0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="B18" s="2">
-        <v>1995.0</v>
-      </c>
-      <c r="C18" s="2">
-        <v>3.0</v>
-      </c>
-      <c r="D18" s="2">
+        <v>104</v>
+      </c>
+      <c r="B18" s="6">
+        <v>1999.0</v>
+      </c>
+      <c r="C18" s="6">
+        <v>9.0</v>
+      </c>
+      <c r="D18" s="6">
         <v>2026.0</v>
       </c>
-      <c r="E18" s="2">
-        <v>88.0</v>
-      </c>
-      <c r="F18" s="2">
+      <c r="E18" s="6">
+        <v>13.0</v>
+      </c>
+      <c r="F18" s="6">
         <v>1.0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="B19" s="2">
-        <v>1997.0</v>
-      </c>
-      <c r="C19" s="2">
-        <v>3.0</v>
-      </c>
-      <c r="D19" s="2">
+        <v>110</v>
+      </c>
+      <c r="B19" s="6">
+        <v>1998.0</v>
+      </c>
+      <c r="C19" s="6">
+        <v>9.0</v>
+      </c>
+      <c r="D19" s="6">
         <v>2026.0</v>
       </c>
-      <c r="E19" s="2">
-        <v>74.0</v>
-      </c>
-      <c r="F19" s="2">
+      <c r="E19" s="6">
+        <v>5.0</v>
+      </c>
+      <c r="F19" s="6">
         <v>1.0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="B20" s="2">
-        <v>2004.0</v>
-      </c>
-      <c r="C20" s="2">
-        <v>3.0</v>
-      </c>
-      <c r="D20" s="2">
+        <v>113</v>
+      </c>
+      <c r="B20" s="6">
+        <v>2003.0</v>
+      </c>
+      <c r="C20" s="6">
+        <v>9.0</v>
+      </c>
+      <c r="D20" s="6">
         <v>2026.0</v>
       </c>
-      <c r="E20" s="2">
-        <v>30.0</v>
-      </c>
-      <c r="F20" s="2">
+      <c r="E20" s="6">
+        <v>35.0</v>
+      </c>
+      <c r="F20" s="6">
         <v>1.0</v>
       </c>
     </row>
@@ -6107,19 +6181,19 @@
       <c r="A21" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="B21" s="2">
-        <v>2004.0</v>
-      </c>
-      <c r="C21" s="2">
-        <v>3.0</v>
-      </c>
-      <c r="D21" s="2">
+      <c r="B21" s="6">
+        <v>2003.0</v>
+      </c>
+      <c r="C21" s="6">
+        <v>9.0</v>
+      </c>
+      <c r="D21" s="6">
         <v>2026.0</v>
       </c>
-      <c r="E21" s="2">
-        <v>26.0</v>
-      </c>
-      <c r="F21" s="2">
+      <c r="E21" s="6">
+        <v>30.0</v>
+      </c>
+      <c r="F21" s="6">
         <v>1.0</v>
       </c>
     </row>
@@ -6127,19 +6201,19 @@
       <c r="A22" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="B22" s="2">
+      <c r="B22" s="6">
         <v>2005.0</v>
       </c>
-      <c r="C22" s="2">
-        <v>3.0</v>
-      </c>
-      <c r="D22" s="2">
+      <c r="C22" s="6">
+        <v>9.0</v>
+      </c>
+      <c r="D22" s="6">
         <v>2026.0</v>
       </c>
-      <c r="E22" s="2">
-        <v>12.0</v>
-      </c>
-      <c r="F22" s="2">
+      <c r="E22" s="6">
+        <v>45.0</v>
+      </c>
+      <c r="F22" s="6">
         <v>1.0</v>
       </c>
     </row>
@@ -6147,46 +6221,502 @@
       <c r="A23" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="B23" s="2">
+      <c r="B23" s="6">
+        <v>1999.0</v>
+      </c>
+      <c r="C23" s="6">
+        <v>6.0</v>
+      </c>
+      <c r="D23" s="6">
+        <v>2026.0</v>
+      </c>
+      <c r="E23" s="6">
+        <v>4.0</v>
+      </c>
+      <c r="F23" s="6">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="A24" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="B24" s="7">
+        <v>2000.0</v>
+      </c>
+      <c r="C24" s="7">
+        <v>6.0</v>
+      </c>
+      <c r="D24" s="7">
+        <v>2026.0</v>
+      </c>
+      <c r="E24" s="7">
+        <v>27.0</v>
+      </c>
+      <c r="F24" s="7">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="A25" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="B25" s="7">
+        <v>2000.0</v>
+      </c>
+      <c r="C25" s="7">
+        <v>6.0</v>
+      </c>
+      <c r="D25" s="7">
+        <v>2026.0</v>
+      </c>
+      <c r="E25" s="7">
+        <v>32.0</v>
+      </c>
+      <c r="F25" s="7">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="26" ht="15.75" customHeight="1">
+      <c r="A26" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="B26" s="7">
+        <v>2002.0</v>
+      </c>
+      <c r="C26" s="8">
+        <v>6.0</v>
+      </c>
+      <c r="D26" s="8">
+        <v>2026.0</v>
+      </c>
+      <c r="E26" s="7">
+        <v>2.0</v>
+      </c>
+      <c r="F26" s="8">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="27" ht="15.75" customHeight="1">
+      <c r="A27" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="B27" s="7">
+        <v>2003.0</v>
+      </c>
+      <c r="C27" s="7">
+        <v>5.0</v>
+      </c>
+      <c r="D27" s="7">
+        <v>2026.0</v>
+      </c>
+      <c r="E27" s="7">
+        <v>108.0</v>
+      </c>
+      <c r="F27" s="7">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="28" ht="15.75" customHeight="1">
+      <c r="A28" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="B28" s="7">
+        <v>1998.0</v>
+      </c>
+      <c r="C28" s="7">
+        <v>5.0</v>
+      </c>
+      <c r="D28" s="7">
+        <v>2026.0</v>
+      </c>
+      <c r="E28" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="F28" s="7">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="29" ht="15.75" customHeight="1">
+      <c r="A29" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="B29" s="7">
+        <v>1995.0</v>
+      </c>
+      <c r="C29" s="7">
+        <v>5.0</v>
+      </c>
+      <c r="D29" s="7">
+        <v>2026.0</v>
+      </c>
+      <c r="E29" s="7">
+        <v>21.0</v>
+      </c>
+      <c r="F29" s="7">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="30" ht="15.75" customHeight="1">
+      <c r="A30" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="B30" s="7">
+        <v>1998.0</v>
+      </c>
+      <c r="C30" s="7">
+        <v>10.0</v>
+      </c>
+      <c r="D30" s="7">
+        <v>2026.0</v>
+      </c>
+      <c r="E30" s="7">
+        <v>5.0</v>
+      </c>
+      <c r="F30" s="7">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="31" ht="15.75" customHeight="1">
+      <c r="A31" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="B31" s="7">
+        <v>2000.0</v>
+      </c>
+      <c r="C31" s="7">
+        <v>10.0</v>
+      </c>
+      <c r="D31" s="7">
+        <v>2026.0</v>
+      </c>
+      <c r="E31" s="7">
+        <v>20.0</v>
+      </c>
+      <c r="F31" s="7">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="32" ht="15.75" customHeight="1">
+      <c r="A32" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="B32" s="7">
+        <v>2000.0</v>
+      </c>
+      <c r="C32" s="7">
+        <v>10.0</v>
+      </c>
+      <c r="D32" s="7">
+        <v>2026.0</v>
+      </c>
+      <c r="E32" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="F32" s="7">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="33" ht="15.75" customHeight="1">
+      <c r="A33" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="B33" s="7">
+        <v>2003.0</v>
+      </c>
+      <c r="C33" s="7">
+        <v>10.0</v>
+      </c>
+      <c r="D33" s="7">
+        <v>2026.0</v>
+      </c>
+      <c r="E33" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="F33" s="7">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="34" ht="15.75" customHeight="1">
+      <c r="A34" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="B34" s="7">
+        <v>1998.0</v>
+      </c>
+      <c r="C34" s="7">
+        <v>7.0</v>
+      </c>
+      <c r="D34" s="7">
+        <v>2026.0</v>
+      </c>
+      <c r="E34" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="F34" s="7">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="35" ht="15.75" customHeight="1">
+      <c r="A35" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="B35" s="7">
+        <v>1999.0</v>
+      </c>
+      <c r="C35" s="7">
+        <v>7.0</v>
+      </c>
+      <c r="D35" s="7">
+        <v>2026.0</v>
+      </c>
+      <c r="E35" s="7">
+        <v>6.0</v>
+      </c>
+      <c r="F35" s="7">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="36" ht="15.75" customHeight="1">
+      <c r="A36" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="B36" s="7">
+        <v>1999.0</v>
+      </c>
+      <c r="C36" s="7">
+        <v>7.0</v>
+      </c>
+      <c r="D36" s="7">
+        <v>2026.0</v>
+      </c>
+      <c r="E36" s="7">
+        <v>35.0</v>
+      </c>
+      <c r="F36" s="7">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="37" ht="15.75" customHeight="1">
+      <c r="A37" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="B37" s="7">
         <v>2005.0</v>
       </c>
-      <c r="C23" s="2">
-        <v>3.0</v>
-      </c>
-      <c r="D23" s="2">
+      <c r="C37" s="7">
+        <v>7.0</v>
+      </c>
+      <c r="D37" s="7">
         <v>2026.0</v>
       </c>
-      <c r="E23" s="2">
-        <v>9.0</v>
-      </c>
-      <c r="F23" s="2">
+      <c r="E37" s="7">
+        <v>7.0</v>
+      </c>
+      <c r="F37" s="7">
         <v>1.0</v>
       </c>
     </row>
-    <row r="24" ht="15.75" customHeight="1"/>
-    <row r="25" ht="15.75" customHeight="1"/>
-    <row r="26" ht="15.75" customHeight="1"/>
-    <row r="27" ht="15.75" customHeight="1"/>
-    <row r="28" ht="15.75" customHeight="1"/>
-    <row r="29" ht="15.75" customHeight="1"/>
-    <row r="30" ht="15.75" customHeight="1"/>
-    <row r="31" ht="15.75" customHeight="1"/>
-    <row r="32" ht="15.75" customHeight="1"/>
-    <row r="33" ht="15.75" customHeight="1"/>
-    <row r="34" ht="15.75" customHeight="1"/>
-    <row r="35" ht="15.75" customHeight="1"/>
-    <row r="36" ht="15.75" customHeight="1"/>
-    <row r="37" ht="15.75" customHeight="1"/>
-    <row r="38" ht="15.75" customHeight="1"/>
-    <row r="39" ht="15.75" customHeight="1"/>
-    <row r="40" ht="15.75" customHeight="1"/>
-    <row r="41" ht="15.75" customHeight="1"/>
-    <row r="42" ht="15.75" customHeight="1"/>
-    <row r="43" ht="15.75" customHeight="1"/>
-    <row r="44" ht="15.75" customHeight="1"/>
-    <row r="45" ht="15.75" customHeight="1"/>
-    <row r="46" ht="15.75" customHeight="1"/>
-    <row r="47" ht="15.75" customHeight="1"/>
+    <row r="38" ht="15.75" customHeight="1">
+      <c r="A38" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="B38" s="7">
+        <v>2000.0</v>
+      </c>
+      <c r="C38" s="7">
+        <v>2.0</v>
+      </c>
+      <c r="D38" s="7">
+        <v>2026.0</v>
+      </c>
+      <c r="E38" s="7">
+        <v>92.0</v>
+      </c>
+      <c r="F38" s="7">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="39" ht="15.75" customHeight="1">
+      <c r="A39" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="B39" s="7">
+        <v>2003.0</v>
+      </c>
+      <c r="C39" s="7">
+        <v>2.0</v>
+      </c>
+      <c r="D39" s="7">
+        <v>2026.0</v>
+      </c>
+      <c r="E39" s="7">
+        <v>50.0</v>
+      </c>
+      <c r="F39" s="7">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="40" ht="15.75" customHeight="1">
+      <c r="A40" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="B40" s="7">
+        <v>1994.0</v>
+      </c>
+      <c r="C40" s="7">
+        <v>2.0</v>
+      </c>
+      <c r="D40" s="7">
+        <v>2026.0</v>
+      </c>
+      <c r="E40" s="7">
+        <v>25.0</v>
+      </c>
+      <c r="F40" s="7">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="41" ht="15.75" customHeight="1">
+      <c r="A41" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="B41" s="7">
+        <v>2004.0</v>
+      </c>
+      <c r="C41" s="7">
+        <v>2.0</v>
+      </c>
+      <c r="D41" s="7">
+        <v>2026.0</v>
+      </c>
+      <c r="E41" s="7">
+        <v>5.0</v>
+      </c>
+      <c r="F41" s="7">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="42" ht="15.75" customHeight="1">
+      <c r="A42" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="B42" s="7">
+        <v>2002.0</v>
+      </c>
+      <c r="C42" s="7">
+        <v>2.0</v>
+      </c>
+      <c r="D42" s="7">
+        <v>2026.0</v>
+      </c>
+      <c r="E42" s="7">
+        <v>31.0</v>
+      </c>
+      <c r="F42" s="7">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="43" ht="15.75" customHeight="1">
+      <c r="A43" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="B43" s="7">
+        <v>1995.0</v>
+      </c>
+      <c r="C43" s="7">
+        <v>2.0</v>
+      </c>
+      <c r="D43" s="7">
+        <v>2026.0</v>
+      </c>
+      <c r="E43" s="7">
+        <v>42.0</v>
+      </c>
+      <c r="F43" s="7">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="44" ht="15.75" customHeight="1">
+      <c r="A44" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="B44" s="7">
+        <v>1996.0</v>
+      </c>
+      <c r="C44" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="D44" s="7">
+        <v>2026.0</v>
+      </c>
+      <c r="E44" s="7">
+        <v>31.0</v>
+      </c>
+      <c r="F44" s="7">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="45" ht="15.75" customHeight="1">
+      <c r="A45" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="B45" s="7">
+        <v>2003.0</v>
+      </c>
+      <c r="C45" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="D45" s="7">
+        <v>2026.0</v>
+      </c>
+      <c r="E45" s="7">
+        <v>11.0</v>
+      </c>
+      <c r="F45" s="7">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="46" ht="15.75" customHeight="1">
+      <c r="A46" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="B46" s="7">
+        <v>2001.0</v>
+      </c>
+      <c r="C46" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="D46" s="7">
+        <v>2026.0</v>
+      </c>
+      <c r="E46" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="F46" s="7">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="47" ht="15.75" customHeight="1">
+      <c r="A47" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="B47" s="7">
+        <v>1997.0</v>
+      </c>
+      <c r="C47" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="D47" s="7">
+        <v>2026.0</v>
+      </c>
+      <c r="E47" s="7">
+        <v>24.0</v>
+      </c>
+      <c r="F47" s="7">
+        <v>1.0</v>
+      </c>
+    </row>
     <row r="48" ht="15.75" customHeight="1"/>
     <row r="49" ht="15.75" customHeight="1"/>
     <row r="50" ht="15.75" customHeight="1"/>
@@ -7164,20 +7694,20 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B1" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="E1" s="7" t="s">
-        <v>81</v>
+      <c r="A1" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -8185,223 +8715,223 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="C1" s="3" t="s">
+      <c r="A1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="F1" s="3" t="s">
+      <c r="D1" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="B2" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="C2" s="3">
+        <v>8.0</v>
+      </c>
+      <c r="D2" s="3">
+        <v>2486.0</v>
+      </c>
+      <c r="E2" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="B3" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="C3" s="3">
+        <v>5.0</v>
+      </c>
+      <c r="D3" s="3">
+        <v>2471.0</v>
+      </c>
+      <c r="E3" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="B4" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="C4" s="3">
+        <v>4.0</v>
+      </c>
+      <c r="D4" s="3">
+        <v>2419.5</v>
+      </c>
+      <c r="E4" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="B5" s="3">
+        <v>4.0</v>
+      </c>
+      <c r="C5" s="3">
+        <v>9.0</v>
+      </c>
+      <c r="D5" s="3">
+        <v>2433.0</v>
+      </c>
+      <c r="E5" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="B6" s="3">
+        <v>5.0</v>
+      </c>
+      <c r="C6" s="3">
+        <v>7.0</v>
+      </c>
+      <c r="D6" s="3">
+        <v>2392.5</v>
+      </c>
+      <c r="E6" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="B7" s="3">
+        <v>6.0</v>
+      </c>
+      <c r="C7" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="D7" s="3">
+        <v>2480.0</v>
+      </c>
+      <c r="E7" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="B8" s="3">
+        <v>7.0</v>
+      </c>
+      <c r="C8" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="D8" s="3">
+        <v>2384.0</v>
+      </c>
+      <c r="E8" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="F8" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2">
+    <row r="9">
+      <c r="A9" s="3">
         <v>2026.0</v>
       </c>
-      <c r="B2" s="2">
-        <v>1.0</v>
-      </c>
-      <c r="C2" s="2">
+      <c r="B9" s="3">
         <v>8.0</v>
       </c>
-      <c r="D2" s="2">
-        <v>2486.0</v>
-      </c>
-      <c r="E2" s="2">
-        <v>1.0</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2">
+      <c r="C9" s="3">
+        <v>10.0</v>
+      </c>
+      <c r="D9" s="3">
+        <v>2396.0</v>
+      </c>
+      <c r="E9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3">
         <v>2026.0</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B10" s="3">
+        <v>9.0</v>
+      </c>
+      <c r="C10" s="3">
         <v>2.0</v>
       </c>
-      <c r="C3" s="2">
-        <v>5.0</v>
-      </c>
-      <c r="D3" s="2">
-        <v>2471.0</v>
-      </c>
-      <c r="E3" s="2">
+      <c r="D10" s="3">
+        <v>2400.0</v>
+      </c>
+      <c r="E10" s="3">
         <v>0.0</v>
       </c>
-      <c r="F3" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2">
+      <c r="F10" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3">
         <v>2026.0</v>
       </c>
-      <c r="B4" s="2">
-        <v>3.0</v>
-      </c>
-      <c r="C4" s="2">
-        <v>4.0</v>
-      </c>
-      <c r="D4" s="2">
-        <v>2419.5</v>
-      </c>
-      <c r="E4" s="2">
+      <c r="B11" s="3">
+        <v>10.0</v>
+      </c>
+      <c r="C11" s="3">
+        <v>6.0</v>
+      </c>
+      <c r="D11" s="3">
+        <v>2395.5</v>
+      </c>
+      <c r="E11" s="3">
         <v>0.0</v>
       </c>
-      <c r="F4" s="2" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2">
-        <v>2026.0</v>
-      </c>
-      <c r="B5" s="2">
-        <v>4.0</v>
-      </c>
-      <c r="C5" s="2">
-        <v>9.0</v>
-      </c>
-      <c r="D5" s="2">
-        <v>2433.0</v>
-      </c>
-      <c r="E5" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2">
-        <v>2026.0</v>
-      </c>
-      <c r="B6" s="2">
-        <v>5.0</v>
-      </c>
-      <c r="C6" s="2">
-        <v>7.0</v>
-      </c>
-      <c r="D6" s="2">
-        <v>2392.5</v>
-      </c>
-      <c r="E6" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2">
-        <v>2026.0</v>
-      </c>
-      <c r="B7" s="2">
-        <v>6.0</v>
-      </c>
-      <c r="C7" s="2">
-        <v>3.0</v>
-      </c>
-      <c r="D7" s="2">
-        <v>2480.0</v>
-      </c>
-      <c r="E7" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2">
-        <v>2026.0</v>
-      </c>
-      <c r="B8" s="2">
-        <v>7.0</v>
-      </c>
-      <c r="C8" s="2">
-        <v>1.0</v>
-      </c>
-      <c r="D8" s="2">
-        <v>2384.0</v>
-      </c>
-      <c r="E8" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2">
-        <v>2026.0</v>
-      </c>
-      <c r="B9" s="2">
-        <v>8.0</v>
-      </c>
-      <c r="C9" s="2">
-        <v>10.0</v>
-      </c>
-      <c r="D9" s="2">
-        <v>2396.0</v>
-      </c>
-      <c r="E9" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2">
-        <v>2026.0</v>
-      </c>
-      <c r="B10" s="2">
-        <v>9.0</v>
-      </c>
-      <c r="C10" s="2">
-        <v>2.0</v>
-      </c>
-      <c r="D10" s="2">
-        <v>2400.0</v>
-      </c>
-      <c r="E10" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2">
-        <v>2026.0</v>
-      </c>
-      <c r="B11" s="2">
-        <v>10.0</v>
-      </c>
-      <c r="C11" s="2">
-        <v>6.0</v>
-      </c>
-      <c r="D11" s="2">
-        <v>2395.5</v>
-      </c>
-      <c r="E11" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>47</v>
+      <c r="F11" s="3" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -9407,45 +9937,45 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="C1" s="3" t="s">
+      <c r="A1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
-        <v>7</v>
+      <c r="D1" s="1" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2">
+      <c r="A2" s="3">
         <v>2026.0</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="3">
         <v>1.0</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="3">
         <v>4.0</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>36</v>
+      <c r="D2" s="3" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2">
+      <c r="A3" s="3">
         <v>2026.0</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="3">
         <v>2.0</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="3">
         <v>8.0</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>59</v>
+      <c r="D3" s="3" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -10450,157 +10980,157 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="B2" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="C2" s="3">
+        <v>32.0</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2">
+    </row>
+    <row r="3">
+      <c r="A3" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="B3" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="C3" s="3">
+        <v>13.0</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="B4" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="C4" s="3">
+        <v>34.0</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3">
+        <v>4.0</v>
+      </c>
+      <c r="B5" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="C5" s="3">
+        <v>10.0</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3">
+        <v>5.0</v>
+      </c>
+      <c r="B6" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="C6" s="3">
         <v>1.0</v>
       </c>
-      <c r="B2" s="2">
+      <c r="D6" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3">
+        <v>6.0</v>
+      </c>
+      <c r="B7" s="3">
         <v>2026.0</v>
       </c>
-      <c r="C2" s="2">
-        <v>32.0</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2">
-        <v>2.0</v>
-      </c>
-      <c r="B3" s="2">
+      <c r="C7" s="3">
+        <v>4.0</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3">
+        <v>7.0</v>
+      </c>
+      <c r="B8" s="3">
         <v>2026.0</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C8" s="3">
+        <v>33.0</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3">
+        <v>8.0</v>
+      </c>
+      <c r="B9" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="C9" s="3">
         <v>13.0</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2">
-        <v>3.0</v>
-      </c>
-      <c r="B4" s="2">
+      <c r="D9" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3">
+        <v>9.0</v>
+      </c>
+      <c r="B10" s="3">
         <v>2026.0</v>
       </c>
-      <c r="C4" s="2">
-        <v>34.0</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2">
-        <v>4.0</v>
-      </c>
-      <c r="B5" s="2">
+      <c r="C10" s="3">
+        <v>14.0</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3">
+        <v>10.0</v>
+      </c>
+      <c r="B11" s="3">
         <v>2026.0</v>
       </c>
-      <c r="C5" s="2">
-        <v>10.0</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2">
-        <v>5.0</v>
-      </c>
-      <c r="B6" s="2">
-        <v>2026.0</v>
-      </c>
-      <c r="C6" s="2">
-        <v>1.0</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2">
-        <v>6.0</v>
-      </c>
-      <c r="B7" s="2">
-        <v>2026.0</v>
-      </c>
-      <c r="C7" s="2">
-        <v>4.0</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2">
-        <v>7.0</v>
-      </c>
-      <c r="B8" s="2">
-        <v>2026.0</v>
-      </c>
-      <c r="C8" s="2">
-        <v>33.0</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2">
-        <v>8.0</v>
-      </c>
-      <c r="B9" s="2">
-        <v>2026.0</v>
-      </c>
-      <c r="C9" s="2">
-        <v>13.0</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2">
-        <v>9.0</v>
-      </c>
-      <c r="B10" s="2">
-        <v>2026.0</v>
-      </c>
-      <c r="C10" s="2">
-        <v>14.0</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2">
-        <v>10.0</v>
-      </c>
-      <c r="B11" s="2">
-        <v>2026.0</v>
-      </c>
-      <c r="C11" s="2">
+      <c r="C11" s="3">
         <v>27.0</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>65</v>
+      <c r="D11" s="3" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -11608,255 +12138,255 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1" s="3" t="s">
+      <c r="A1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="B2" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2">
+      <c r="D2" s="3">
+        <v>-5.0</v>
+      </c>
+      <c r="E2" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="F2" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="G2" s="3">
+        <v>1027.0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3">
         <v>2026.0</v>
       </c>
-      <c r="B2" s="2">
-        <v>1.0</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D2" s="2">
-        <v>-5.0</v>
-      </c>
-      <c r="E2" s="2">
+      <c r="B3" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="3">
+        <v>-15.0</v>
+      </c>
+      <c r="E3" s="3">
         <v>0.0</v>
       </c>
-      <c r="F2" s="2">
+      <c r="F3" s="3">
         <v>0.0</v>
       </c>
-      <c r="G2" s="2">
-        <v>1027.0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2">
+      <c r="G3" s="3">
+        <v>998.0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3">
         <v>2026.0</v>
       </c>
-      <c r="B3" s="2">
-        <v>2.0</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D3" s="2">
-        <v>-15.0</v>
-      </c>
-      <c r="E3" s="2">
+      <c r="B4" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="3">
         <v>0.0</v>
       </c>
-      <c r="F3" s="2">
+      <c r="E4" s="3">
         <v>0.0</v>
       </c>
-      <c r="G3" s="2">
-        <v>998.0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2">
+      <c r="F4" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="G4" s="3">
+        <v>1034.0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3">
         <v>2026.0</v>
       </c>
-      <c r="B4" s="2">
-        <v>3.0</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D4" s="2">
+      <c r="B5" s="3">
+        <v>4.0</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="3">
+        <v>10.0</v>
+      </c>
+      <c r="E5" s="3">
+        <v>10.0</v>
+      </c>
+      <c r="F5" s="3">
         <v>0.0</v>
       </c>
-      <c r="E4" s="2">
+      <c r="G5" s="3">
+        <v>1030.0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="B6" s="3">
+        <v>5.0</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="3">
+        <v>15.0</v>
+      </c>
+      <c r="E6" s="3">
         <v>0.0</v>
       </c>
-      <c r="F4" s="2">
+      <c r="F6" s="3">
         <v>0.0</v>
       </c>
-      <c r="G4" s="2">
-        <v>1034.0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2">
+      <c r="G6" s="3">
+        <v>1016.0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3">
         <v>2026.0</v>
       </c>
-      <c r="B5" s="2">
-        <v>4.0</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D5" s="2">
+      <c r="B7" s="3">
+        <v>6.0</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="3">
+        <v>-20.0</v>
+      </c>
+      <c r="E7" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="F7" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="G7" s="3">
+        <v>984.0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="B8" s="3">
+        <v>7.0</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="E8" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="F8" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="G8" s="3">
+        <v>1033.0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="B9" s="3">
+        <v>8.0</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D9" s="3">
+        <v>25.0</v>
+      </c>
+      <c r="E9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="F9" s="3">
         <v>10.0</v>
       </c>
-      <c r="E5" s="2">
+      <c r="G9" s="3">
+        <v>1048.0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="B10" s="3">
+        <v>9.0</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D10" s="3">
+        <v>5.0</v>
+      </c>
+      <c r="E10" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="F10" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="G10" s="3">
+        <v>1019.0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="B11" s="3">
         <v>10.0</v>
       </c>
-      <c r="F5" s="2">
+      <c r="C11" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="3">
+        <v>-10.0</v>
+      </c>
+      <c r="E11" s="3">
         <v>0.0</v>
       </c>
-      <c r="G5" s="2">
-        <v>1030.0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2">
-        <v>2026.0</v>
-      </c>
-      <c r="B6" s="2">
-        <v>5.0</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D6" s="2">
-        <v>15.0</v>
-      </c>
-      <c r="E6" s="2">
+      <c r="F11" s="3">
         <v>0.0</v>
       </c>
-      <c r="F6" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="G6" s="2">
-        <v>1016.0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2">
-        <v>2026.0</v>
-      </c>
-      <c r="B7" s="2">
-        <v>6.0</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="D7" s="2">
-        <v>-20.0</v>
-      </c>
-      <c r="E7" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="F7" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="G7" s="2">
-        <v>984.0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2">
-        <v>2026.0</v>
-      </c>
-      <c r="B8" s="2">
-        <v>7.0</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="D8" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="E8" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="F8" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="G8" s="2">
-        <v>1033.0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2">
-        <v>2026.0</v>
-      </c>
-      <c r="B9" s="2">
-        <v>8.0</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D9" s="2">
-        <v>25.0</v>
-      </c>
-      <c r="E9" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="F9" s="2">
-        <v>10.0</v>
-      </c>
-      <c r="G9" s="2">
-        <v>1048.0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2">
-        <v>2026.0</v>
-      </c>
-      <c r="B10" s="2">
-        <v>9.0</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="D10" s="2">
-        <v>5.0</v>
-      </c>
-      <c r="E10" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="F10" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="G10" s="2">
-        <v>1019.0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2">
-        <v>2026.0</v>
-      </c>
-      <c r="B11" s="2">
-        <v>10.0</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="D11" s="2">
-        <v>-10.0</v>
-      </c>
-      <c r="E11" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="F11" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="G11" s="2">
+      <c r="G11" s="3">
         <v>1017.0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Contratti: via Baturina, Malen a 218
Turetta rinuncia a Baturina; corretto il prezzo di Malen.
45 contratti attivi.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dati/Gestione.xlsx
+++ b/dati/Gestione.xlsx
@@ -18,14 +18,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId14" roundtripDataChecksum="B4dhXUFeEllg8s0q66B85rfSqIsn1f5u0SsG7tAXXGo="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId14" roundtripDataChecksum="29Coqi8Je0gsWALXoirptNQv4R3w7kLXuMpx8d5Ytv8="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="169">
   <si>
     <t>FANTA BRECCIA — foglio di gestione</t>
   </si>
@@ -33,348 +33,348 @@
     <t>ID</t>
   </si>
   <si>
+    <t>Questo file e' la fonte unica dei dati del sito.</t>
+  </si>
+  <si>
+    <t>Dopo averlo modificato e SALVATO: doppio click su aggiorna.bat</t>
+  </si>
+  <si>
+    <t>Allenatore</t>
+  </si>
+  <si>
+    <t>Foglio</t>
+  </si>
+  <si>
+    <t>Squadra</t>
+  </si>
+  <si>
+    <t>Tabella SQLite</t>
+  </si>
+  <si>
+    <t>Contenuto</t>
+  </si>
+  <si>
+    <t>AnagraficaSquadre</t>
+  </si>
+  <si>
+    <t>teams</t>
+  </si>
+  <si>
+    <t>Squadre e allenatori (qui stanno gli ID)</t>
+  </si>
+  <si>
+    <t>CambioNome</t>
+  </si>
+  <si>
+    <t>cambio_nome</t>
+  </si>
+  <si>
+    <t>Nome della squadra per anno</t>
+  </si>
+  <si>
+    <t>Contratti</t>
+  </si>
+  <si>
+    <t>contracts + players</t>
+  </si>
+  <si>
+    <t>Contratti di riconferma</t>
+  </si>
+  <si>
+    <t>Svincoli</t>
+  </si>
+  <si>
+    <t>contract_releases</t>
+  </si>
+  <si>
+    <t>Svincoli: storico e penali</t>
+  </si>
+  <si>
+    <t>Classifiche</t>
+  </si>
+  <si>
+    <t>season_rankings</t>
+  </si>
+  <si>
+    <t>Classifica di campionato</t>
+  </si>
+  <si>
+    <t>Coppa</t>
+  </si>
+  <si>
+    <t>coppa</t>
+  </si>
+  <si>
+    <t>Podio della coppa</t>
+  </si>
+  <si>
+    <t>Anno</t>
+  </si>
+  <si>
+    <t>CreditiAsta</t>
+  </si>
+  <si>
+    <t>credit_residual</t>
+  </si>
+  <si>
+    <t>Crediti avanzati a fine stagione</t>
+  </si>
+  <si>
+    <t>Nome</t>
+  </si>
+  <si>
+    <t>CreditiAnnoNuovo</t>
+  </si>
+  <si>
+    <t>Mindo</t>
+  </si>
+  <si>
+    <t>crediti_anno_nuovo</t>
+  </si>
+  <si>
+    <t>Budget della stagione nuova</t>
+  </si>
+  <si>
     <t>Giocatore</t>
   </si>
   <si>
-    <t>Allenatore</t>
-  </si>
-  <si>
-    <t>Squadra</t>
-  </si>
-  <si>
-    <t>Questo file e' la fonte unica dei dati del sito.</t>
-  </si>
-  <si>
-    <t>Mindo</t>
-  </si>
-  <si>
     <t>Chentus</t>
   </si>
   <si>
-    <t>Dopo averlo modificato e SALVATO: doppio click su aggiorna.bat</t>
+    <t>FOGLIO CONTRATTI</t>
   </si>
   <si>
     <t>Alessio Cocchieri &amp; Febio</t>
   </si>
   <si>
-    <t>Anno</t>
+    <t>nome del calciatore, scritto per esteso</t>
   </si>
   <si>
     <t>MALLOREDDUS FC</t>
   </si>
   <si>
-    <t>Foglio</t>
+    <t>AnnoNascita</t>
+  </si>
+  <si>
+    <t>solo l'anno: da qui dipende la categoria A/B/C</t>
+  </si>
+  <si>
+    <t>Sporting Garra</t>
+  </si>
+  <si>
+    <t>IDSquadra</t>
+  </si>
+  <si>
+    <t>ID come in AnagraficaSquadre</t>
   </si>
   <si>
     <t>PietroPJ</t>
   </si>
   <si>
-    <t>Sporting Garra</t>
-  </si>
-  <si>
-    <t>Nome</t>
+    <t>Whiteam FC</t>
+  </si>
+  <si>
+    <t>AnnoInizio</t>
+  </si>
+  <si>
+    <t>anno della riconferma</t>
+  </si>
+  <si>
+    <t>PrezzoAcquisto</t>
+  </si>
+  <si>
+    <t>TurettaEPacciani FC</t>
+  </si>
+  <si>
+    <t>prezzo pagato all'asta: non cambia mai</t>
   </si>
   <si>
     <t>Max Allegri</t>
   </si>
   <si>
-    <t>Whiteam FC</t>
-  </si>
-  <si>
-    <t>AnnoNascita</t>
+    <t>Nkunku Settete</t>
+  </si>
+  <si>
+    <t>Attivo</t>
+  </si>
+  <si>
+    <t>1 se in corso, 0 se chiuso</t>
   </si>
   <si>
     <t>Fil e Pacciansss &amp; sono innocenti</t>
   </si>
   <si>
-    <t>TurettaEPacciani FC</t>
-  </si>
-  <si>
-    <t>Tabella SQLite</t>
+    <t>Mapi Group</t>
+  </si>
+  <si>
+    <t>ANNO FINE NON SI SCRIVE</t>
+  </si>
+  <si>
+    <t>e' sempre AnnoInizio + 3 (regolamento par. 1)</t>
+  </si>
+  <si>
+    <t>Roul e il socio</t>
+  </si>
+  <si>
+    <t>FOGLIO SVINCOLI</t>
+  </si>
+  <si>
+    <t>Compagnia Ascolana Sigari</t>
+  </si>
+  <si>
+    <t>stesso nome scritto in Contratti</t>
   </si>
   <si>
     <t>Alessio Bruni</t>
   </si>
   <si>
-    <t>IDSquadra</t>
-  </si>
-  <si>
-    <t>Nkunku Settete</t>
-  </si>
-  <si>
-    <t>Contenuto</t>
-  </si>
-  <si>
-    <t>AnnoInizio</t>
+    <t>Tridente demoniaco</t>
+  </si>
+  <si>
+    <t>Davis K.</t>
+  </si>
+  <si>
+    <t>la squadra che lo svincola</t>
+  </si>
+  <si>
+    <t>AnnoSvincolo</t>
   </si>
   <si>
     <t>deiu &amp; Bep</t>
   </si>
   <si>
-    <t>Mapi Group</t>
-  </si>
-  <si>
-    <t>PrezzoAcquisto</t>
-  </si>
-  <si>
-    <t>AnagraficaSquadre</t>
-  </si>
-  <si>
-    <t>teams</t>
-  </si>
-  <si>
-    <t>Attivo</t>
+    <t>anno in cui viene svincolato</t>
+  </si>
+  <si>
+    <t>Penale</t>
+  </si>
+  <si>
+    <t>LASCIALA VUOTA: la calcola il sistema.</t>
+  </si>
+  <si>
+    <t>Compilala solo per forzare un valore diverso.</t>
   </si>
   <si>
     <t>CariBam &amp; sickroul</t>
   </si>
   <si>
-    <t>Squadre e allenatori (qui stanno gli ID)</t>
-  </si>
-  <si>
-    <t>Roul e il socio</t>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>motivo, facoltativo</t>
+  </si>
+  <si>
+    <t>Thorstvedt</t>
+  </si>
+  <si>
+    <t>QUANDO SVINCOLI UN GIOCATORE</t>
   </si>
   <si>
     <t>Luca baffi e tabacchi</t>
   </si>
   <si>
-    <t>Davis K.</t>
-  </si>
-  <si>
-    <t>CambioNome</t>
-  </si>
-  <si>
-    <t>Compagnia Ascolana Sigari</t>
-  </si>
-  <si>
-    <t>cambio_nome</t>
-  </si>
-  <si>
-    <t>Nome della squadra per anno</t>
+    <t>1. Aggiungi la riga qui in Svincoli</t>
+  </si>
+  <si>
+    <t>2. Metti Attivo = 0 nella sua riga di Contratti</t>
+  </si>
+  <si>
+    <t>La penale viene tolta dai crediti dell'asta successiva.</t>
   </si>
   <si>
     <t>mister zeman</t>
   </si>
   <si>
-    <t>Tridente demoniaco</t>
-  </si>
-  <si>
-    <t>Contratti</t>
-  </si>
-  <si>
-    <t>contracts + players</t>
-  </si>
-  <si>
-    <t>Contratti di riconferma</t>
-  </si>
-  <si>
-    <t>Thorstvedt</t>
-  </si>
-  <si>
-    <t>Svincoli</t>
-  </si>
-  <si>
-    <t>contract_releases</t>
-  </si>
-  <si>
-    <t>Svincoli: storico e penali</t>
-  </si>
-  <si>
-    <t>Classifiche</t>
-  </si>
-  <si>
-    <t>season_rankings</t>
-  </si>
-  <si>
-    <t>Classifica di campionato</t>
-  </si>
-  <si>
     <t>Da Cunha</t>
   </si>
   <si>
-    <t>Coppa</t>
-  </si>
-  <si>
-    <t>coppa</t>
-  </si>
-  <si>
-    <t>Podio della coppa</t>
-  </si>
-  <si>
-    <t>CreditiAsta</t>
+    <t>CATEGORIE (sull'anno di riferimento)</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>eta' &lt;= 21</t>
+  </si>
+  <si>
+    <t>illimitati</t>
   </si>
   <si>
     <t>Samardzic</t>
   </si>
   <si>
-    <t>credit_residual</t>
-  </si>
-  <si>
-    <t>Crediti avanzati a fine stagione</t>
-  </si>
-  <si>
-    <t>CreditiAnnoNuovo</t>
-  </si>
-  <si>
-    <t>crediti_anno_nuovo</t>
-  </si>
-  <si>
-    <t>Budget della stagione nuova</t>
+    <t>B</t>
+  </si>
+  <si>
+    <t>eta' &lt;= 25</t>
+  </si>
+  <si>
+    <t>nessun limite proprio, ma A+B &lt;= 6</t>
   </si>
   <si>
     <t>Ghilardi</t>
   </si>
   <si>
-    <t>FOGLIO CONTRATTI</t>
-  </si>
-  <si>
-    <t>nome del calciatore, scritto per esteso</t>
+    <t>A</t>
+  </si>
+  <si>
+    <t>oltre i 25</t>
   </si>
   <si>
     <t>Vlasic</t>
   </si>
   <si>
-    <t>solo l'anno: da qui dipende la categoria A/B/C</t>
-  </si>
-  <si>
-    <t>ID come in AnagraficaSquadre</t>
+    <t>massimo 3</t>
+  </si>
+  <si>
+    <t>CREDITI DELLA STAGIONE NUOVA</t>
+  </si>
+  <si>
+    <t>Non si compilano a mano.</t>
+  </si>
+  <si>
+    <t>strumenti\calcola_crediti.py li calcola</t>
   </si>
   <si>
     <t>Lauriente</t>
   </si>
   <si>
-    <t>anno della riconferma</t>
-  </si>
-  <si>
     <t>Bisseck</t>
   </si>
   <si>
-    <t>prezzo pagato all'asta: non cambia mai</t>
-  </si>
-  <si>
     <t>Rowe</t>
   </si>
   <si>
-    <t>1 se in corso, 0 se chiuso</t>
-  </si>
-  <si>
-    <t>ANNO FINE NON SI SCRIVE</t>
-  </si>
-  <si>
-    <t>e' sempre AnnoInizio + 3 (regolamento par. 1)</t>
-  </si>
-  <si>
     <t>Rodriguez Je.</t>
   </si>
   <si>
-    <t>FOGLIO SVINCOLI</t>
-  </si>
-  <si>
-    <t>stesso nome scritto in Contratti</t>
-  </si>
-  <si>
     <t>Bernasconi</t>
   </si>
   <si>
-    <t>la squadra che lo svincola</t>
-  </si>
-  <si>
-    <t>AnnoSvincolo</t>
-  </si>
-  <si>
-    <t>anno in cui viene svincolato</t>
-  </si>
-  <si>
     <t>Ramon</t>
   </si>
   <si>
-    <t>Penale</t>
-  </si>
-  <si>
-    <t>LASCIALA VUOTA: la calcola il sistema.</t>
-  </si>
-  <si>
     <t>Dimarco</t>
   </si>
   <si>
-    <t>Compilala solo per forzare un valore diverso.</t>
-  </si>
-  <si>
-    <t>Note</t>
-  </si>
-  <si>
-    <t>motivo, facoltativo</t>
-  </si>
-  <si>
     <t>Gaetano</t>
   </si>
   <si>
-    <t>QUANDO SVINCOLI UN GIOCATORE</t>
-  </si>
-  <si>
-    <t>1. Aggiungi la riga qui in Svincoli</t>
-  </si>
-  <si>
     <t>Malen</t>
   </si>
   <si>
-    <t>2. Metti Attivo = 0 nella sua riga di Contratti</t>
-  </si>
-  <si>
-    <t>La penale viene tolta dai crediti dell'asta successiva.</t>
-  </si>
-  <si>
-    <t>CATEGORIE (sull'anno di riferimento)</t>
-  </si>
-  <si>
     <t>Douvikas</t>
   </si>
   <si>
-    <t>C</t>
-  </si>
-  <si>
-    <t>eta' &lt;= 21</t>
-  </si>
-  <si>
-    <t>illimitati</t>
-  </si>
-  <si>
     <t>Frattesi</t>
   </si>
   <si>
-    <t>B</t>
-  </si>
-  <si>
-    <t>eta' &lt;= 25</t>
-  </si>
-  <si>
-    <t>nessun limite proprio, ma A+B &lt;= 6</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>oltre i 25</t>
-  </si>
-  <si>
     <t>Martinez Jo.</t>
   </si>
   <si>
-    <t>massimo 3</t>
-  </si>
-  <si>
-    <t>CREDITI DELLA STAGIONE NUOVA</t>
-  </si>
-  <si>
     <t>Bonny</t>
   </si>
   <si>
-    <t>Non si compilano a mano.</t>
-  </si>
-  <si>
-    <t>strumenti\calcola_crediti.py li calcola</t>
-  </si>
-  <si>
     <t>Atta</t>
   </si>
   <si>
@@ -393,9 +393,6 @@
     <t>Belghali</t>
   </si>
   <si>
-    <t>Baturina</t>
-  </si>
-  <si>
     <t>McKennie</t>
   </si>
   <si>
@@ -435,12 +432,21 @@
     <t>Rrahmani</t>
   </si>
   <si>
+    <t>Posizione</t>
+  </si>
+  <si>
     <t>Valle</t>
   </si>
   <si>
+    <t>Punteggio</t>
+  </si>
+  <si>
     <t>Colombo</t>
   </si>
   <si>
+    <t>Miglior Punteggio</t>
+  </si>
+  <si>
     <t>Simeone</t>
   </si>
   <si>
@@ -454,15 +460,6 @@
   </si>
   <si>
     <t>Dovbyk</t>
-  </si>
-  <si>
-    <t>Posizione</t>
-  </si>
-  <si>
-    <t>Punteggio</t>
-  </si>
-  <si>
-    <t>Miglior Punteggio</t>
   </si>
   <si>
     <t>CreditiFineAnno</t>
@@ -550,14 +547,14 @@
     </font>
     <font>
       <b/>
-      <sz val="11.0"/>
-      <color rgb="FFFFFFFF"/>
+      <sz val="14.0"/>
+      <color rgb="FF7A3E12"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="14.0"/>
-      <color rgb="FF7A3E12"/>
+      <sz val="11.0"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -628,15 +625,15 @@
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="1" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
@@ -646,10 +643,10 @@
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" vertical="bottom"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -908,303 +905,303 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>8</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>38</v>
+        <v>12</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>40</v>
+        <v>13</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>41</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>44</v>
+        <v>15</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>45</v>
+        <v>16</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>46</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>48</v>
+        <v>18</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>49</v>
+        <v>19</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>50</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>51</v>
+        <v>21</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>52</v>
+        <v>22</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>53</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>55</v>
+        <v>24</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>57</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>58</v>
+        <v>28</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>60</v>
+        <v>29</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>61</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>62</v>
+        <v>32</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>63</v>
+        <v>34</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>64</v>
+        <v>35</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="s">
-        <v>66</v>
+      <c r="A16" s="4" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="s">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>67</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>69</v>
+        <v>43</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>70</v>
+        <v>46</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>26</v>
+        <v>49</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>72</v>
+        <v>50</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="3" t="s">
-        <v>29</v>
+        <v>51</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>74</v>
+        <v>53</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="3" t="s">
-        <v>32</v>
+        <v>56</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>76</v>
+        <v>57</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="3" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>78</v>
+        <v>61</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1"/>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="5" t="s">
-        <v>80</v>
+      <c r="A25" s="4" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="3" t="s">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>81</v>
+        <v>65</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="3" t="s">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="3" t="s">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>85</v>
+        <v>72</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="3" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>88</v>
+        <v>74</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="C30" s="3" t="s">
-        <v>90</v>
+        <v>75</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="3" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1"/>
     <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="5" t="s">
-        <v>94</v>
+      <c r="A33" s="4" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="3" t="s">
-        <v>95</v>
+        <v>82</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="3" t="s">
-        <v>97</v>
+        <v>83</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="3" t="s">
-        <v>98</v>
+        <v>84</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1"/>
     <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="5" t="s">
-        <v>99</v>
+      <c r="A38" s="4" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="3" t="s">
-        <v>101</v>
+        <v>88</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>102</v>
+        <v>89</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>103</v>
+        <v>90</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="3" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="3" t="s">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1"/>
     <row r="43" ht="15.75" customHeight="1">
-      <c r="A43" s="5" t="s">
-        <v>112</v>
+      <c r="A43" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="3" t="s">
-        <v>114</v>
+        <v>101</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>115</v>
+        <v>102</v>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1"/>
@@ -2189,27 +2186,27 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="C1" s="10" t="s">
         <v>151</v>
       </c>
-      <c r="B1" s="10" t="s">
-        <v>143</v>
-      </c>
-      <c r="C1" s="10" t="s">
+      <c r="D1" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="E1" s="10" t="s">
         <v>152</v>
       </c>
-      <c r="D1" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="E1" s="10" t="s">
+      <c r="F1" s="10" t="s">
         <v>153</v>
-      </c>
-      <c r="F1" s="10" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C2" s="3">
         <v>1000.0</v>
@@ -2221,12 +2218,12 @@
         <v>2999.0</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C3" s="3">
         <v>950.0</v>
@@ -2238,12 +2235,12 @@
         <v>2999.0</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C4" s="3">
         <v>1100.0</v>
@@ -2255,12 +2252,12 @@
         <v>2999.0</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C5" s="3">
         <v>900.0</v>
@@ -2272,12 +2269,12 @@
         <v>2999.0</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B6" s="3">
         <v>1.0</v>
@@ -2292,12 +2289,12 @@
         <v>2999.0</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B7" s="3">
         <v>2.0</v>
@@ -2312,12 +2309,12 @@
         <v>2999.0</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B8" s="3">
         <v>3.0</v>
@@ -2332,12 +2329,12 @@
         <v>2999.0</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B9" s="3">
         <v>4.0</v>
@@ -2352,12 +2349,12 @@
         <v>2999.0</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B10" s="3">
         <v>5.0</v>
@@ -2372,12 +2369,12 @@
         <v>2999.0</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B11" s="3">
         <v>6.0</v>
@@ -2392,12 +2389,12 @@
         <v>2999.0</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B12" s="3">
         <v>7.0</v>
@@ -2412,12 +2409,12 @@
         <v>2999.0</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B13" s="3">
         <v>8.0</v>
@@ -2432,12 +2429,12 @@
         <v>2999.0</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B14" s="3">
         <v>9.0</v>
@@ -2452,12 +2449,12 @@
         <v>2999.0</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B15" s="3">
         <v>10.0</v>
@@ -2472,12 +2469,12 @@
         <v>2999.0</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C16" s="3">
         <v>10.0</v>
@@ -2489,12 +2486,12 @@
         <v>2999.0</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="s">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="C17" s="3">
         <v>10.0</v>
@@ -2506,12 +2503,12 @@
         <v>2999.0</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C18" s="3">
         <v>50.0</v>
@@ -2523,7 +2520,7 @@
         <v>2999.0</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -3528,14 +3525,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>4</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="2">
@@ -3543,10 +3540,10 @@
         <v>1.0</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>7</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3">
@@ -3554,10 +3551,10 @@
         <v>2.0</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>9</v>
+        <v>39</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>11</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4">
@@ -3565,10 +3562,10 @@
         <v>3.0</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>13</v>
+        <v>47</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>14</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5">
@@ -3576,10 +3573,10 @@
         <v>4.0</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>16</v>
+        <v>54</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>17</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6">
@@ -3587,10 +3584,10 @@
         <v>5.0</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>19</v>
+        <v>58</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>20</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7">
@@ -3598,10 +3595,10 @@
         <v>6.0</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>24</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8">
@@ -3609,10 +3606,10 @@
         <v>7.0</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>27</v>
+        <v>71</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>28</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9">
@@ -3620,10 +3617,10 @@
         <v>8.0</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>33</v>
+        <v>76</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>35</v>
+        <v>62</v>
       </c>
     </row>
     <row r="10">
@@ -3631,10 +3628,10 @@
         <v>9.0</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>36</v>
+        <v>81</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>39</v>
+        <v>64</v>
       </c>
     </row>
     <row r="11">
@@ -3642,10 +3639,10 @@
         <v>10.0</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>42</v>
+        <v>85</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>43</v>
+        <v>67</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -4649,14 +4646,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>15</v>
+      <c r="B1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="2">
@@ -4667,7 +4664,7 @@
         <v>2026.0</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>7</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3">
@@ -4678,7 +4675,7 @@
         <v>2026.0</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>11</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4">
@@ -4689,7 +4686,7 @@
         <v>2026.0</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>14</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5">
@@ -4700,7 +4697,7 @@
         <v>2026.0</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>17</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6">
@@ -4711,7 +4708,7 @@
         <v>2026.0</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>20</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7">
@@ -4722,7 +4719,7 @@
         <v>2026.0</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>24</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8">
@@ -4733,7 +4730,7 @@
         <v>2026.0</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>28</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9">
@@ -4744,7 +4741,7 @@
         <v>2026.0</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>35</v>
+        <v>62</v>
       </c>
     </row>
     <row r="10">
@@ -4755,7 +4752,7 @@
         <v>2026.0</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>39</v>
+        <v>64</v>
       </c>
     </row>
     <row r="11">
@@ -4766,7 +4763,7 @@
         <v>2026.0</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>43</v>
+        <v>67</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -5773,28 +5770,28 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>32</v>
+      <c r="A1" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="s">
-        <v>37</v>
+        <v>68</v>
       </c>
       <c r="B2" s="6">
         <v>1998.0</v>
@@ -5814,7 +5811,7 @@
     </row>
     <row r="3">
       <c r="A3" s="6" t="s">
-        <v>47</v>
+        <v>79</v>
       </c>
       <c r="B3" s="6">
         <v>1999.0</v>
@@ -5835,7 +5832,7 @@
     </row>
     <row r="4">
       <c r="A4" s="6" t="s">
-        <v>54</v>
+        <v>86</v>
       </c>
       <c r="B4" s="6">
         <v>2001.0</v>
@@ -5856,7 +5853,7 @@
     </row>
     <row r="5">
       <c r="A5" s="6" t="s">
-        <v>59</v>
+        <v>91</v>
       </c>
       <c r="B5" s="6">
         <v>2002.0</v>
@@ -5877,7 +5874,7 @@
     </row>
     <row r="6">
       <c r="A6" s="6" t="s">
-        <v>65</v>
+        <v>95</v>
       </c>
       <c r="B6" s="6">
         <v>2003.0</v>
@@ -5898,7 +5895,7 @@
     </row>
     <row r="7">
       <c r="A7" s="6" t="s">
-        <v>68</v>
+        <v>98</v>
       </c>
       <c r="B7" s="6">
         <v>1997.0</v>
@@ -5919,7 +5916,7 @@
     </row>
     <row r="8">
       <c r="A8" s="6" t="s">
-        <v>71</v>
+        <v>103</v>
       </c>
       <c r="B8" s="6">
         <v>1998.0</v>
@@ -5939,7 +5936,7 @@
     </row>
     <row r="9">
       <c r="A9" s="6" t="s">
-        <v>73</v>
+        <v>104</v>
       </c>
       <c r="B9" s="6">
         <v>2000.0</v>
@@ -5959,7 +5956,7 @@
     </row>
     <row r="10">
       <c r="A10" s="6" t="s">
-        <v>75</v>
+        <v>105</v>
       </c>
       <c r="B10" s="6">
         <v>2003.0</v>
@@ -5979,7 +5976,7 @@
     </row>
     <row r="11">
       <c r="A11" s="6" t="s">
-        <v>79</v>
+        <v>106</v>
       </c>
       <c r="B11" s="6">
         <v>2005.0</v>
@@ -5999,7 +5996,7 @@
     </row>
     <row r="12">
       <c r="A12" s="6" t="s">
-        <v>82</v>
+        <v>107</v>
       </c>
       <c r="B12" s="6">
         <v>2003.0</v>
@@ -6019,7 +6016,7 @@
     </row>
     <row r="13">
       <c r="A13" s="6" t="s">
-        <v>86</v>
+        <v>108</v>
       </c>
       <c r="B13" s="6">
         <v>2005.0</v>
@@ -6039,7 +6036,7 @@
     </row>
     <row r="14">
       <c r="A14" s="6" t="s">
-        <v>89</v>
+        <v>109</v>
       </c>
       <c r="B14" s="6">
         <v>1997.0</v>
@@ -6059,7 +6056,7 @@
     </row>
     <row r="15">
       <c r="A15" s="6" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="B15" s="6">
         <v>2000.0</v>
@@ -6079,7 +6076,7 @@
     </row>
     <row r="16">
       <c r="A16" s="6" t="s">
-        <v>96</v>
+        <v>111</v>
       </c>
       <c r="B16" s="6">
         <v>1999.0</v>
@@ -6091,7 +6088,7 @@
         <v>2026.0</v>
       </c>
       <c r="E16" s="6">
-        <v>210.0</v>
+        <v>218.0</v>
       </c>
       <c r="F16" s="6">
         <v>1.0</v>
@@ -6099,7 +6096,7 @@
     </row>
     <row r="17">
       <c r="A17" s="6" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="B17" s="6">
         <v>1999.0</v>
@@ -6119,7 +6116,7 @@
     </row>
     <row r="18">
       <c r="A18" s="6" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="B18" s="6">
         <v>1999.0</v>
@@ -6139,7 +6136,7 @@
     </row>
     <row r="19">
       <c r="A19" s="6" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B19" s="6">
         <v>1998.0</v>
@@ -6159,7 +6156,7 @@
     </row>
     <row r="20">
       <c r="A20" s="6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B20" s="6">
         <v>2003.0</v>
@@ -6302,7 +6299,7 @@
         <v>122</v>
       </c>
       <c r="B27" s="7">
-        <v>2003.0</v>
+        <v>1998.0</v>
       </c>
       <c r="C27" s="7">
         <v>5.0</v>
@@ -6311,7 +6308,7 @@
         <v>2026.0</v>
       </c>
       <c r="E27" s="7">
-        <v>108.0</v>
+        <v>1.0</v>
       </c>
       <c r="F27" s="7">
         <v>1.0</v>
@@ -6322,7 +6319,7 @@
         <v>123</v>
       </c>
       <c r="B28" s="7">
-        <v>1998.0</v>
+        <v>1995.0</v>
       </c>
       <c r="C28" s="7">
         <v>5.0</v>
@@ -6331,7 +6328,7 @@
         <v>2026.0</v>
       </c>
       <c r="E28" s="7">
-        <v>1.0</v>
+        <v>21.0</v>
       </c>
       <c r="F28" s="7">
         <v>1.0</v>
@@ -6342,16 +6339,16 @@
         <v>124</v>
       </c>
       <c r="B29" s="7">
-        <v>1995.0</v>
+        <v>1998.0</v>
       </c>
       <c r="C29" s="7">
-        <v>5.0</v>
+        <v>10.0</v>
       </c>
       <c r="D29" s="7">
         <v>2026.0</v>
       </c>
       <c r="E29" s="7">
-        <v>21.0</v>
+        <v>5.0</v>
       </c>
       <c r="F29" s="7">
         <v>1.0</v>
@@ -6362,7 +6359,7 @@
         <v>125</v>
       </c>
       <c r="B30" s="7">
-        <v>1998.0</v>
+        <v>2000.0</v>
       </c>
       <c r="C30" s="7">
         <v>10.0</v>
@@ -6371,7 +6368,7 @@
         <v>2026.0</v>
       </c>
       <c r="E30" s="7">
-        <v>5.0</v>
+        <v>20.0</v>
       </c>
       <c r="F30" s="7">
         <v>1.0</v>
@@ -6391,7 +6388,7 @@
         <v>2026.0</v>
       </c>
       <c r="E31" s="7">
-        <v>20.0</v>
+        <v>1.0</v>
       </c>
       <c r="F31" s="7">
         <v>1.0</v>
@@ -6402,7 +6399,7 @@
         <v>127</v>
       </c>
       <c r="B32" s="7">
-        <v>2000.0</v>
+        <v>2003.0</v>
       </c>
       <c r="C32" s="7">
         <v>10.0</v>
@@ -6422,10 +6419,10 @@
         <v>128</v>
       </c>
       <c r="B33" s="7">
-        <v>2003.0</v>
+        <v>1998.0</v>
       </c>
       <c r="C33" s="7">
-        <v>10.0</v>
+        <v>7.0</v>
       </c>
       <c r="D33" s="7">
         <v>2026.0</v>
@@ -6442,7 +6439,7 @@
         <v>129</v>
       </c>
       <c r="B34" s="7">
-        <v>1998.0</v>
+        <v>1999.0</v>
       </c>
       <c r="C34" s="7">
         <v>7.0</v>
@@ -6451,7 +6448,7 @@
         <v>2026.0</v>
       </c>
       <c r="E34" s="7">
-        <v>1.0</v>
+        <v>6.0</v>
       </c>
       <c r="F34" s="7">
         <v>1.0</v>
@@ -6471,7 +6468,7 @@
         <v>2026.0</v>
       </c>
       <c r="E35" s="7">
-        <v>6.0</v>
+        <v>35.0</v>
       </c>
       <c r="F35" s="7">
         <v>1.0</v>
@@ -6482,7 +6479,7 @@
         <v>131</v>
       </c>
       <c r="B36" s="7">
-        <v>1999.0</v>
+        <v>2005.0</v>
       </c>
       <c r="C36" s="7">
         <v>7.0</v>
@@ -6491,7 +6488,7 @@
         <v>2026.0</v>
       </c>
       <c r="E36" s="7">
-        <v>35.0</v>
+        <v>7.0</v>
       </c>
       <c r="F36" s="7">
         <v>1.0</v>
@@ -6502,16 +6499,16 @@
         <v>132</v>
       </c>
       <c r="B37" s="7">
-        <v>2005.0</v>
+        <v>2000.0</v>
       </c>
       <c r="C37" s="7">
-        <v>7.0</v>
+        <v>2.0</v>
       </c>
       <c r="D37" s="7">
         <v>2026.0</v>
       </c>
       <c r="E37" s="7">
-        <v>7.0</v>
+        <v>92.0</v>
       </c>
       <c r="F37" s="7">
         <v>1.0</v>
@@ -6522,7 +6519,7 @@
         <v>133</v>
       </c>
       <c r="B38" s="7">
-        <v>2000.0</v>
+        <v>2003.0</v>
       </c>
       <c r="C38" s="7">
         <v>2.0</v>
@@ -6531,7 +6528,7 @@
         <v>2026.0</v>
       </c>
       <c r="E38" s="7">
-        <v>92.0</v>
+        <v>50.0</v>
       </c>
       <c r="F38" s="7">
         <v>1.0</v>
@@ -6542,7 +6539,7 @@
         <v>134</v>
       </c>
       <c r="B39" s="7">
-        <v>2003.0</v>
+        <v>1994.0</v>
       </c>
       <c r="C39" s="7">
         <v>2.0</v>
@@ -6551,7 +6548,7 @@
         <v>2026.0</v>
       </c>
       <c r="E39" s="7">
-        <v>50.0</v>
+        <v>25.0</v>
       </c>
       <c r="F39" s="7">
         <v>1.0</v>
@@ -6559,10 +6556,10 @@
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="7" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B40" s="7">
-        <v>1994.0</v>
+        <v>2004.0</v>
       </c>
       <c r="C40" s="7">
         <v>2.0</v>
@@ -6571,7 +6568,7 @@
         <v>2026.0</v>
       </c>
       <c r="E40" s="7">
-        <v>25.0</v>
+        <v>5.0</v>
       </c>
       <c r="F40" s="7">
         <v>1.0</v>
@@ -6579,10 +6576,10 @@
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="7" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B41" s="7">
-        <v>2004.0</v>
+        <v>2002.0</v>
       </c>
       <c r="C41" s="7">
         <v>2.0</v>
@@ -6591,7 +6588,7 @@
         <v>2026.0</v>
       </c>
       <c r="E41" s="7">
-        <v>5.0</v>
+        <v>31.0</v>
       </c>
       <c r="F41" s="7">
         <v>1.0</v>
@@ -6599,10 +6596,10 @@
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="7" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B42" s="7">
-        <v>2002.0</v>
+        <v>1995.0</v>
       </c>
       <c r="C42" s="7">
         <v>2.0</v>
@@ -6611,7 +6608,7 @@
         <v>2026.0</v>
       </c>
       <c r="E42" s="7">
-        <v>31.0</v>
+        <v>42.0</v>
       </c>
       <c r="F42" s="7">
         <v>1.0</v>
@@ -6619,19 +6616,19 @@
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="7" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B43" s="7">
-        <v>1995.0</v>
+        <v>1996.0</v>
       </c>
       <c r="C43" s="7">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="D43" s="7">
         <v>2026.0</v>
       </c>
       <c r="E43" s="7">
-        <v>42.0</v>
+        <v>31.0</v>
       </c>
       <c r="F43" s="7">
         <v>1.0</v>
@@ -6639,10 +6636,10 @@
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="7" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B44" s="7">
-        <v>1996.0</v>
+        <v>2003.0</v>
       </c>
       <c r="C44" s="7">
         <v>1.0</v>
@@ -6651,7 +6648,7 @@
         <v>2026.0</v>
       </c>
       <c r="E44" s="7">
-        <v>31.0</v>
+        <v>11.0</v>
       </c>
       <c r="F44" s="7">
         <v>1.0</v>
@@ -6659,10 +6656,10 @@
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="7" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="B45" s="7">
-        <v>2003.0</v>
+        <v>2001.0</v>
       </c>
       <c r="C45" s="7">
         <v>1.0</v>
@@ -6671,7 +6668,7 @@
         <v>2026.0</v>
       </c>
       <c r="E45" s="7">
-        <v>11.0</v>
+        <v>1.0</v>
       </c>
       <c r="F45" s="7">
         <v>1.0</v>
@@ -6679,10 +6676,10 @@
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="7" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B46" s="7">
-        <v>2001.0</v>
+        <v>1997.0</v>
       </c>
       <c r="C46" s="7">
         <v>1.0</v>
@@ -6691,32 +6688,13 @@
         <v>2026.0</v>
       </c>
       <c r="E46" s="7">
-        <v>1.0</v>
+        <v>24.0</v>
       </c>
       <c r="F46" s="7">
         <v>1.0</v>
       </c>
     </row>
-    <row r="47" ht="15.75" customHeight="1">
-      <c r="A47" s="7" t="s">
-        <v>142</v>
-      </c>
-      <c r="B47" s="7">
-        <v>1997.0</v>
-      </c>
-      <c r="C47" s="7">
-        <v>1.0</v>
-      </c>
-      <c r="D47" s="7">
-        <v>2026.0</v>
-      </c>
-      <c r="E47" s="7">
-        <v>24.0</v>
-      </c>
-      <c r="F47" s="7">
-        <v>1.0</v>
-      </c>
-    </row>
+    <row r="47" ht="15.75" customHeight="1"/>
     <row r="48" ht="15.75" customHeight="1"/>
     <row r="49" ht="15.75" customHeight="1"/>
     <row r="50" ht="15.75" customHeight="1"/>
@@ -7669,7 +7647,6 @@
     <row r="997" ht="15.75" customHeight="1"/>
     <row r="998" ht="15.75" customHeight="1"/>
     <row r="999" ht="15.75" customHeight="1"/>
-    <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <printOptions/>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
@@ -7695,19 +7672,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="9" t="s">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -8715,23 +8692,23 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>4</v>
+      <c r="D1" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="2">
@@ -8751,7 +8728,7 @@
         <v>1.0</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>35</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3">
@@ -8771,7 +8748,7 @@
         <v>0.0</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>20</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4">
@@ -8791,7 +8768,7 @@
         <v>0.0</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>17</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5">
@@ -8811,7 +8788,7 @@
         <v>0.0</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>39</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6">
@@ -8831,7 +8808,7 @@
         <v>0.0</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>28</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7">
@@ -8851,7 +8828,7 @@
         <v>0.0</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>14</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8">
@@ -8871,7 +8848,7 @@
         <v>0.0</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>7</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9">
@@ -8891,7 +8868,7 @@
         <v>0.0</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>43</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10">
@@ -8911,7 +8888,7 @@
         <v>0.0</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>11</v>
+        <v>41</v>
       </c>
     </row>
     <row r="11">
@@ -8931,7 +8908,7 @@
         <v>0.0</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>24</v>
+        <v>55</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -9937,17 +9914,17 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>4</v>
+      <c r="D1" s="2" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="2">
@@ -9961,7 +9938,7 @@
         <v>4.0</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>17</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3">
@@ -9975,7 +9952,7 @@
         <v>8.0</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>35</v>
+        <v>62</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -10980,17 +10957,17 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>15</v>
+      <c r="B1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="2">
@@ -11004,7 +10981,7 @@
         <v>32.0</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3">
@@ -11018,7 +10995,7 @@
         <v>13.0</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>9</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4">
@@ -11032,7 +11009,7 @@
         <v>34.0</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>13</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5">
@@ -11046,7 +11023,7 @@
         <v>10.0</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>16</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6">
@@ -11060,7 +11037,7 @@
         <v>1.0</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>19</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7">
@@ -11074,7 +11051,7 @@
         <v>4.0</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>22</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8">
@@ -11088,7 +11065,7 @@
         <v>33.0</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>27</v>
+        <v>71</v>
       </c>
     </row>
     <row r="9">
@@ -11102,7 +11079,7 @@
         <v>13.0</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>33</v>
+        <v>76</v>
       </c>
     </row>
     <row r="10">
@@ -11116,7 +11093,7 @@
         <v>14.0</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>36</v>
+        <v>81</v>
       </c>
     </row>
     <row r="11">
@@ -11130,7 +11107,7 @@
         <v>27.0</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>42</v>
+        <v>85</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -12138,26 +12115,26 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="C1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>149</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="2">
@@ -12168,7 +12145,7 @@
         <v>1.0</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>7</v>
+        <v>37</v>
       </c>
       <c r="D2" s="3">
         <v>-5.0</v>
@@ -12191,7 +12168,7 @@
         <v>2.0</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>11</v>
+        <v>41</v>
       </c>
       <c r="D3" s="3">
         <v>-15.0</v>
@@ -12214,7 +12191,7 @@
         <v>3.0</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>14</v>
+        <v>44</v>
       </c>
       <c r="D4" s="3">
         <v>0.0</v>
@@ -12237,7 +12214,7 @@
         <v>4.0</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>17</v>
+        <v>48</v>
       </c>
       <c r="D5" s="3">
         <v>10.0</v>
@@ -12260,7 +12237,7 @@
         <v>5.0</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>20</v>
+        <v>52</v>
       </c>
       <c r="D6" s="3">
         <v>15.0</v>
@@ -12283,7 +12260,7 @@
         <v>6.0</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>24</v>
+        <v>55</v>
       </c>
       <c r="D7" s="3">
         <v>-20.0</v>
@@ -12306,7 +12283,7 @@
         <v>7.0</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>28</v>
+        <v>59</v>
       </c>
       <c r="D8" s="3">
         <v>0.0</v>
@@ -12329,7 +12306,7 @@
         <v>8.0</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>35</v>
+        <v>62</v>
       </c>
       <c r="D9" s="3">
         <v>25.0</v>
@@ -12352,7 +12329,7 @@
         <v>9.0</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>39</v>
+        <v>64</v>
       </c>
       <c r="D10" s="3">
         <v>5.0</v>
@@ -12375,7 +12352,7 @@
         <v>10.0</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>43</v>
+        <v>67</v>
       </c>
       <c r="D11" s="3">
         <v>-10.0</v>

</xml_diff>

<commit_message>
Contratti: Bernasconi a 10
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dati/Gestione.xlsx
+++ b/dati/Gestione.xlsx
@@ -27,51 +27,138 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="169">
   <si>
+    <t>ID</t>
+  </si>
+  <si>
     <t>FANTA BRECCIA — foglio di gestione</t>
   </si>
   <si>
-    <t>ID</t>
+    <t>Allenatore</t>
+  </si>
+  <si>
+    <t>Squadra</t>
+  </si>
+  <si>
+    <t>Anno</t>
   </si>
   <si>
     <t>Questo file e' la fonte unica dei dati del sito.</t>
   </si>
   <si>
+    <t>Giocatore</t>
+  </si>
+  <si>
+    <t>Mindo</t>
+  </si>
+  <si>
+    <t>Chentus</t>
+  </si>
+  <si>
     <t>Dopo averlo modificato e SALVATO: doppio click su aggiorna.bat</t>
   </si>
   <si>
-    <t>Allenatore</t>
+    <t>Alessio Cocchieri &amp; Febio</t>
+  </si>
+  <si>
+    <t>MALLOREDDUS FC</t>
   </si>
   <si>
     <t>Foglio</t>
   </si>
   <si>
-    <t>Squadra</t>
+    <t>PietroPJ</t>
+  </si>
+  <si>
+    <t>Sporting Garra</t>
+  </si>
+  <si>
+    <t>Max Allegri</t>
+  </si>
+  <si>
+    <t>Whiteam FC</t>
+  </si>
+  <si>
+    <t>AnnoNascita</t>
+  </si>
+  <si>
+    <t>Fil e Pacciansss &amp; sono innocenti</t>
+  </si>
+  <si>
+    <t>TurettaEPacciani FC</t>
   </si>
   <si>
     <t>Tabella SQLite</t>
   </si>
   <si>
+    <t>Alessio Bruni</t>
+  </si>
+  <si>
+    <t>IDSquadra</t>
+  </si>
+  <si>
+    <t>Nkunku Settete</t>
+  </si>
+  <si>
     <t>Contenuto</t>
   </si>
   <si>
+    <t>deiu &amp; Bep</t>
+  </si>
+  <si>
+    <t>Mapi Group</t>
+  </si>
+  <si>
+    <t>AnnoInizio</t>
+  </si>
+  <si>
     <t>AnagraficaSquadre</t>
   </si>
   <si>
+    <t>CariBam &amp; sickraoul</t>
+  </si>
+  <si>
+    <t>Nome</t>
+  </si>
+  <si>
+    <t>Raoul e il socio</t>
+  </si>
+  <si>
     <t>teams</t>
   </si>
   <si>
+    <t>PrezzoAcquisto</t>
+  </si>
+  <si>
     <t>Squadre e allenatori (qui stanno gli ID)</t>
   </si>
   <si>
+    <t>Luca baffi e tabacchi</t>
+  </si>
+  <si>
+    <t>Compagnia Ascolana Sigari</t>
+  </si>
+  <si>
+    <t>Attivo</t>
+  </si>
+  <si>
     <t>CambioNome</t>
   </si>
   <si>
+    <t>mister zeman</t>
+  </si>
+  <si>
     <t>cambio_nome</t>
   </si>
   <si>
+    <t>Tridente demoniaco</t>
+  </si>
+  <si>
     <t>Nome della squadra per anno</t>
   </si>
   <si>
+    <t>Davis K.</t>
+  </si>
+  <si>
     <t>Contratti</t>
   </si>
   <si>
@@ -87,6 +174,9 @@
     <t>contract_releases</t>
   </si>
   <si>
+    <t>Thorstvedt</t>
+  </si>
+  <si>
     <t>Svincoli: storico e penali</t>
   </si>
   <si>
@@ -105,12 +195,12 @@
     <t>coppa</t>
   </si>
   <si>
+    <t>Da Cunha</t>
+  </si>
+  <si>
     <t>Podio della coppa</t>
   </si>
   <si>
-    <t>Anno</t>
-  </si>
-  <si>
     <t>CreditiAsta</t>
   </si>
   <si>
@@ -120,118 +210,67 @@
     <t>Crediti avanzati a fine stagione</t>
   </si>
   <si>
-    <t>Nome</t>
-  </si>
-  <si>
     <t>CreditiAnnoNuovo</t>
   </si>
   <si>
-    <t>Mindo</t>
-  </si>
-  <si>
     <t>crediti_anno_nuovo</t>
   </si>
   <si>
+    <t>Samardzic</t>
+  </si>
+  <si>
     <t>Budget della stagione nuova</t>
   </si>
   <si>
-    <t>Giocatore</t>
-  </si>
-  <si>
-    <t>Chentus</t>
-  </si>
-  <si>
     <t>FOGLIO CONTRATTI</t>
   </si>
   <si>
-    <t>Alessio Cocchieri &amp; Febio</t>
+    <t>Ghilardi</t>
+  </si>
+  <si>
+    <t>Vlasic</t>
   </si>
   <si>
     <t>nome del calciatore, scritto per esteso</t>
   </si>
   <si>
-    <t>MALLOREDDUS FC</t>
-  </si>
-  <si>
-    <t>AnnoNascita</t>
-  </si>
-  <si>
     <t>solo l'anno: da qui dipende la categoria A/B/C</t>
   </si>
   <si>
-    <t>Sporting Garra</t>
-  </si>
-  <si>
-    <t>IDSquadra</t>
-  </si>
-  <si>
     <t>ID come in AnagraficaSquadre</t>
   </si>
   <si>
-    <t>PietroPJ</t>
-  </si>
-  <si>
-    <t>Whiteam FC</t>
-  </si>
-  <si>
-    <t>AnnoInizio</t>
+    <t>Lauriente</t>
   </si>
   <si>
     <t>anno della riconferma</t>
   </si>
   <si>
-    <t>PrezzoAcquisto</t>
-  </si>
-  <si>
-    <t>TurettaEPacciani FC</t>
+    <t>Bisseck</t>
   </si>
   <si>
     <t>prezzo pagato all'asta: non cambia mai</t>
   </si>
   <si>
-    <t>Max Allegri</t>
-  </si>
-  <si>
-    <t>Nkunku Settete</t>
-  </si>
-  <si>
-    <t>Attivo</t>
-  </si>
-  <si>
     <t>1 se in corso, 0 se chiuso</t>
   </si>
   <si>
-    <t>Fil e Pacciansss &amp; sono innocenti</t>
-  </si>
-  <si>
-    <t>Mapi Group</t>
-  </si>
-  <si>
     <t>ANNO FINE NON SI SCRIVE</t>
   </si>
   <si>
     <t>e' sempre AnnoInizio + 3 (regolamento par. 1)</t>
   </si>
   <si>
-    <t>Raoul e il socio</t>
+    <t>Rowe</t>
   </si>
   <si>
     <t>FOGLIO SVINCOLI</t>
   </si>
   <si>
-    <t>Compagnia Ascolana Sigari</t>
-  </si>
-  <si>
     <t>stesso nome scritto in Contratti</t>
   </si>
   <si>
-    <t>Alessio Bruni</t>
-  </si>
-  <si>
-    <t>Tridente demoniaco</t>
-  </si>
-  <si>
-    <t>Davis K.</t>
+    <t>Rodriguez Je.</t>
   </si>
   <si>
     <t>la squadra che lo svincola</t>
@@ -240,12 +279,12 @@
     <t>AnnoSvincolo</t>
   </si>
   <si>
-    <t>deiu &amp; Bep</t>
-  </si>
-  <si>
     <t>anno in cui viene svincolato</t>
   </si>
   <si>
+    <t>Bernasconi</t>
+  </si>
+  <si>
     <t>Penale</t>
   </si>
   <si>
@@ -255,42 +294,36 @@
     <t>Compilala solo per forzare un valore diverso.</t>
   </si>
   <si>
-    <t>CariBam &amp; sickraoul</t>
-  </si>
-  <si>
     <t>Note</t>
   </si>
   <si>
     <t>motivo, facoltativo</t>
   </si>
   <si>
-    <t>Thorstvedt</t>
+    <t>Ramon</t>
   </si>
   <si>
     <t>QUANDO SVINCOLI UN GIOCATORE</t>
   </si>
   <si>
-    <t>Luca baffi e tabacchi</t>
-  </si>
-  <si>
     <t>1. Aggiungi la riga qui in Svincoli</t>
   </si>
   <si>
     <t>2. Metti Attivo = 0 nella sua riga di Contratti</t>
   </si>
   <si>
+    <t>Dimarco</t>
+  </si>
+  <si>
     <t>La penale viene tolta dai crediti dell'asta successiva.</t>
   </si>
   <si>
-    <t>mister zeman</t>
-  </si>
-  <si>
-    <t>Da Cunha</t>
-  </si>
-  <si>
     <t>CATEGORIE (sull'anno di riferimento)</t>
   </si>
   <si>
+    <t>Gaetano</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
@@ -300,33 +333,30 @@
     <t>illimitati</t>
   </si>
   <si>
-    <t>Samardzic</t>
-  </si>
-  <si>
     <t>B</t>
   </si>
   <si>
     <t>eta' &lt;= 25</t>
   </si>
   <si>
+    <t>Malen</t>
+  </si>
+  <si>
     <t>nessun limite proprio, ma A+B &lt;= 6</t>
   </si>
   <si>
-    <t>Ghilardi</t>
-  </si>
-  <si>
     <t>A</t>
   </si>
   <si>
     <t>oltre i 25</t>
   </si>
   <si>
-    <t>Vlasic</t>
-  </si>
-  <si>
     <t>massimo 3</t>
   </si>
   <si>
+    <t>Douvikas</t>
+  </si>
+  <si>
     <t>CREDITI DELLA STAGIONE NUOVA</t>
   </si>
   <si>
@@ -336,36 +366,6 @@
     <t>strumenti\calcola_crediti.py li calcola</t>
   </si>
   <si>
-    <t>Lauriente</t>
-  </si>
-  <si>
-    <t>Bisseck</t>
-  </si>
-  <si>
-    <t>Rowe</t>
-  </si>
-  <si>
-    <t>Rodriguez Je.</t>
-  </si>
-  <si>
-    <t>Bernasconi</t>
-  </si>
-  <si>
-    <t>Ramon</t>
-  </si>
-  <si>
-    <t>Dimarco</t>
-  </si>
-  <si>
-    <t>Gaetano</t>
-  </si>
-  <si>
-    <t>Malen</t>
-  </si>
-  <si>
-    <t>Douvikas</t>
-  </si>
-  <si>
     <t>Frattesi</t>
   </si>
   <si>
@@ -432,25 +432,25 @@
     <t>Rrahmani</t>
   </si>
   <si>
+    <t>Valle</t>
+  </si>
+  <si>
+    <t>Colombo</t>
+  </si>
+  <si>
     <t>Posizione</t>
   </si>
   <si>
-    <t>Valle</t>
+    <t>Simeone</t>
   </si>
   <si>
     <t>Punteggio</t>
   </si>
   <si>
-    <t>Colombo</t>
+    <t>Mancini</t>
   </si>
   <si>
     <t>Miglior Punteggio</t>
-  </si>
-  <si>
-    <t>Simeone</t>
-  </si>
-  <si>
-    <t>Mancini</t>
   </si>
   <si>
     <t>Casadei</t>
@@ -538,7 +538,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -547,14 +547,14 @@
     </font>
     <font>
       <b/>
-      <sz val="14.0"/>
-      <color rgb="FF7A3E12"/>
+      <sz val="11.0"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="11.0"/>
-      <color rgb="FFFFFFFF"/>
+      <sz val="14.0"/>
+      <color rgb="FF7A3E12"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -565,11 +565,6 @@
       <b/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11.0"/>
@@ -621,32 +616,29 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="1" fillId="2" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf borderId="1" fillId="2" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="1" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" vertical="bottom"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="1" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="5" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -905,303 +897,303 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
+      <c r="A1" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>8</v>
+      <c r="A6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>14</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>15</v>
+        <v>44</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>16</v>
+        <v>45</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>17</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>18</v>
+        <v>47</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>19</v>
+        <v>48</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>20</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>23</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>26</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>28</v>
+        <v>58</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>29</v>
+        <v>59</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>30</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>32</v>
+        <v>61</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>34</v>
+        <v>62</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>35</v>
+        <v>64</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="s">
-        <v>38</v>
+      <c r="A16" s="5" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="s">
-        <v>36</v>
+        <v>6</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>40</v>
+        <v>68</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="s">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>43</v>
+        <v>69</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>46</v>
+        <v>70</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>49</v>
+        <v>27</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>50</v>
+        <v>72</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="3" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>53</v>
+        <v>74</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="3" t="s">
-        <v>56</v>
+        <v>37</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="3" t="s">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>61</v>
+        <v>77</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1"/>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="4" t="s">
-        <v>63</v>
+      <c r="A25" s="5" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="3" t="s">
-        <v>36</v>
+        <v>6</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>65</v>
+        <v>80</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="3" t="s">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="3" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>72</v>
+        <v>84</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="3" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>74</v>
+        <v>87</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="C30" s="3" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="3" t="s">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1"/>
     <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="4" t="s">
-        <v>80</v>
+      <c r="A33" s="5" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="3" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="3" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="3" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1"/>
     <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="4" t="s">
-        <v>87</v>
+      <c r="A38" s="5" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="3" t="s">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="3" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>94</v>
+        <v>105</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="3" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1"/>
     <row r="43" ht="15.75" customHeight="1">
-      <c r="A43" s="4" t="s">
-        <v>100</v>
+      <c r="A43" s="5" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="3" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1"/>
@@ -2185,22 +2177,22 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="9" t="s">
         <v>150</v>
       </c>
-      <c r="B1" s="10" t="s">
-        <v>135</v>
-      </c>
-      <c r="C1" s="10" t="s">
+      <c r="B1" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="C1" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="D1" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="E1" s="10" t="s">
+      <c r="D1" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="F1" s="9" t="s">
         <v>153</v>
       </c>
     </row>
@@ -2491,7 +2483,7 @@
     </row>
     <row r="17">
       <c r="A17" s="3" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="C17" s="3">
         <v>10.0</v>
@@ -3525,14 +3517,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>6</v>
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="2">
@@ -3540,10 +3532,10 @@
         <v>1.0</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>33</v>
+        <v>7</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>37</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3">
@@ -3551,10 +3543,10 @@
         <v>2.0</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>41</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4">
@@ -3562,10 +3554,10 @@
         <v>3.0</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>47</v>
+        <v>13</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5">
@@ -3573,10 +3565,10 @@
         <v>4.0</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>54</v>
+        <v>15</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>48</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6">
@@ -3584,10 +3576,10 @@
         <v>5.0</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>58</v>
+        <v>18</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>52</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7">
@@ -3595,10 +3587,10 @@
         <v>6.0</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>66</v>
+        <v>21</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>55</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8">
@@ -3606,10 +3598,10 @@
         <v>7.0</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>71</v>
+        <v>25</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>59</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9">
@@ -3617,10 +3609,10 @@
         <v>8.0</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>76</v>
+        <v>29</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>62</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10">
@@ -3628,10 +3620,10 @@
         <v>9.0</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>81</v>
+        <v>35</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>64</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11">
@@ -3639,10 +3631,10 @@
         <v>10.0</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>85</v>
+        <v>39</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>67</v>
+        <v>41</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -4646,14 +4638,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>31</v>
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="2">
@@ -4664,7 +4656,7 @@
         <v>2026.0</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>37</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3">
@@ -4675,7 +4667,7 @@
         <v>2026.0</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>41</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4">
@@ -4686,7 +4678,7 @@
         <v>2026.0</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5">
@@ -4697,7 +4689,7 @@
         <v>2026.0</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>48</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6">
@@ -4708,7 +4700,7 @@
         <v>2026.0</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>52</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7">
@@ -4719,7 +4711,7 @@
         <v>2026.0</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>55</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8">
@@ -4730,7 +4722,7 @@
         <v>2026.0</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>59</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9">
@@ -4741,7 +4733,7 @@
         <v>2026.0</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>62</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10">
@@ -4752,7 +4744,7 @@
         <v>2026.0</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>64</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11">
@@ -4763,7 +4755,7 @@
         <v>2026.0</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>67</v>
+        <v>41</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -5770,515 +5762,515 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="D1" s="5" t="s">
+      <c r="A1" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2" s="3">
+        <v>1998.0</v>
+      </c>
+      <c r="C2" s="3">
+        <v>4.0</v>
+      </c>
+      <c r="D2" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="E2" s="3">
+        <v>33.0</v>
+      </c>
+      <c r="F2" s="3">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E1" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="F1" s="5" t="s">
+      <c r="B3" s="3">
+        <v>1999.0</v>
+      </c>
+      <c r="C3" s="3">
+        <v>4.0</v>
+      </c>
+      <c r="D3" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="E3" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="F3" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="I3" s="3"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="B2" s="6">
+      <c r="B4" s="3">
+        <v>2001.0</v>
+      </c>
+      <c r="C4" s="3">
+        <v>4.0</v>
+      </c>
+      <c r="D4" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="E4" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="F4" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="I4" s="3"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B5" s="3">
+        <v>2002.0</v>
+      </c>
+      <c r="C5" s="3">
+        <v>4.0</v>
+      </c>
+      <c r="D5" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="E5" s="3">
+        <v>14.0</v>
+      </c>
+      <c r="F5" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="I5" s="3"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B6" s="3">
+        <v>2003.0</v>
+      </c>
+      <c r="C6" s="3">
+        <v>4.0</v>
+      </c>
+      <c r="D6" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="E6" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="F6" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="I6" s="3"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B7" s="3">
+        <v>1997.0</v>
+      </c>
+      <c r="C7" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="D7" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="E7" s="3">
+        <v>41.0</v>
+      </c>
+      <c r="F7" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="I7" s="3"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B8" s="3">
         <v>1998.0</v>
       </c>
-      <c r="C2" s="6">
+      <c r="C8" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="D8" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="E8" s="3">
+        <v>43.0</v>
+      </c>
+      <c r="F8" s="3">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B9" s="3">
+        <v>2000.0</v>
+      </c>
+      <c r="C9" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="D9" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="E9" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="F9" s="3">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B10" s="3">
+        <v>2003.0</v>
+      </c>
+      <c r="C10" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="D10" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="E10" s="3">
+        <v>17.0</v>
+      </c>
+      <c r="F10" s="3">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B11" s="3">
+        <v>2005.0</v>
+      </c>
+      <c r="C11" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="D11" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="E11" s="3">
+        <v>6.0</v>
+      </c>
+      <c r="F11" s="3">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B12" s="3">
+        <v>2003.0</v>
+      </c>
+      <c r="C12" s="3">
+        <v>8.0</v>
+      </c>
+      <c r="D12" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="E12" s="6">
+        <v>10.0</v>
+      </c>
+      <c r="F12" s="3">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B13" s="3">
+        <v>2005.0</v>
+      </c>
+      <c r="C13" s="3">
+        <v>8.0</v>
+      </c>
+      <c r="D13" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="E13" s="3">
+        <v>10.0</v>
+      </c>
+      <c r="F13" s="3">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B14" s="3">
+        <v>1997.0</v>
+      </c>
+      <c r="C14" s="3">
+        <v>8.0</v>
+      </c>
+      <c r="D14" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="E14" s="3">
+        <v>73.0</v>
+      </c>
+      <c r="F14" s="3">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="B15" s="3">
+        <v>2000.0</v>
+      </c>
+      <c r="C15" s="3">
+        <v>8.0</v>
+      </c>
+      <c r="D15" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="E15" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="F15" s="3">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B16" s="3">
+        <v>1999.0</v>
+      </c>
+      <c r="C16" s="3">
+        <v>8.0</v>
+      </c>
+      <c r="D16" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="E16" s="3">
+        <v>218.0</v>
+      </c>
+      <c r="F16" s="3">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B17" s="3">
+        <v>1999.0</v>
+      </c>
+      <c r="C17" s="3">
+        <v>9.0</v>
+      </c>
+      <c r="D17" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="E17" s="3">
+        <v>24.0</v>
+      </c>
+      <c r="F17" s="3">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="B18" s="3">
+        <v>1999.0</v>
+      </c>
+      <c r="C18" s="3">
+        <v>9.0</v>
+      </c>
+      <c r="D18" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="E18" s="3">
+        <v>13.0</v>
+      </c>
+      <c r="F18" s="3">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="B19" s="3">
+        <v>1998.0</v>
+      </c>
+      <c r="C19" s="3">
+        <v>9.0</v>
+      </c>
+      <c r="D19" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="E19" s="3">
+        <v>5.0</v>
+      </c>
+      <c r="F19" s="3">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B20" s="3">
+        <v>2003.0</v>
+      </c>
+      <c r="C20" s="3">
+        <v>9.0</v>
+      </c>
+      <c r="D20" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="E20" s="3">
+        <v>35.0</v>
+      </c>
+      <c r="F20" s="3">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="B21" s="3">
+        <v>2003.0</v>
+      </c>
+      <c r="C21" s="3">
+        <v>9.0</v>
+      </c>
+      <c r="D21" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="E21" s="3">
+        <v>30.0</v>
+      </c>
+      <c r="F21" s="3">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B22" s="3">
+        <v>2005.0</v>
+      </c>
+      <c r="C22" s="3">
+        <v>9.0</v>
+      </c>
+      <c r="D22" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="E22" s="3">
+        <v>45.0</v>
+      </c>
+      <c r="F22" s="3">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B23" s="3">
+        <v>1999.0</v>
+      </c>
+      <c r="C23" s="3">
+        <v>6.0</v>
+      </c>
+      <c r="D23" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="E23" s="3">
         <v>4.0</v>
       </c>
-      <c r="D2" s="6">
+      <c r="F23" s="3">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="A24" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="B24" s="3">
+        <v>2000.0</v>
+      </c>
+      <c r="C24" s="3">
+        <v>6.0</v>
+      </c>
+      <c r="D24" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E2" s="6">
-        <v>33.0</v>
-      </c>
-      <c r="F2" s="6">
+      <c r="E24" s="3">
+        <v>27.0</v>
+      </c>
+      <c r="F24" s="3">
         <v>1.0</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="B3" s="6">
-        <v>1999.0</v>
-      </c>
-      <c r="C3" s="6">
-        <v>4.0</v>
-      </c>
-      <c r="D3" s="6">
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="A25" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="B25" s="3">
+        <v>2000.0</v>
+      </c>
+      <c r="C25" s="3">
+        <v>6.0</v>
+      </c>
+      <c r="D25" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E3" s="6">
+      <c r="E25" s="3">
+        <v>32.0</v>
+      </c>
+      <c r="F25" s="3">
         <v>1.0</v>
       </c>
-      <c r="F3" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="I3" s="3"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="B4" s="6">
-        <v>2001.0</v>
-      </c>
-      <c r="C4" s="6">
-        <v>4.0</v>
-      </c>
-      <c r="D4" s="6">
-        <v>2026.0</v>
-      </c>
-      <c r="E4" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="F4" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="I4" s="3"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="B5" s="6">
-        <v>2002.0</v>
-      </c>
-      <c r="C5" s="6">
-        <v>4.0</v>
-      </c>
-      <c r="D5" s="6">
-        <v>2026.0</v>
-      </c>
-      <c r="E5" s="6">
-        <v>14.0</v>
-      </c>
-      <c r="F5" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="I5" s="3"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="B6" s="6">
-        <v>2003.0</v>
-      </c>
-      <c r="C6" s="6">
-        <v>4.0</v>
-      </c>
-      <c r="D6" s="6">
-        <v>2026.0</v>
-      </c>
-      <c r="E6" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="F6" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="I6" s="3"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B7" s="6">
-        <v>1997.0</v>
-      </c>
-      <c r="C7" s="6">
-        <v>3.0</v>
-      </c>
-      <c r="D7" s="6">
-        <v>2026.0</v>
-      </c>
-      <c r="E7" s="6">
-        <v>41.0</v>
-      </c>
-      <c r="F7" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="I7" s="3"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="B8" s="6">
-        <v>1998.0</v>
-      </c>
-      <c r="C8" s="6">
-        <v>3.0</v>
-      </c>
-      <c r="D8" s="6">
-        <v>2026.0</v>
-      </c>
-      <c r="E8" s="6">
-        <v>43.0</v>
-      </c>
-      <c r="F8" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="B9" s="6">
-        <v>2000.0</v>
-      </c>
-      <c r="C9" s="6">
-        <v>3.0</v>
-      </c>
-      <c r="D9" s="6">
-        <v>2026.0</v>
-      </c>
-      <c r="E9" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="F9" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="B10" s="6">
-        <v>2003.0</v>
-      </c>
-      <c r="C10" s="6">
-        <v>3.0</v>
-      </c>
-      <c r="D10" s="6">
-        <v>2026.0</v>
-      </c>
-      <c r="E10" s="6">
-        <v>17.0</v>
-      </c>
-      <c r="F10" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="B11" s="6">
-        <v>2005.0</v>
-      </c>
-      <c r="C11" s="6">
-        <v>3.0</v>
-      </c>
-      <c r="D11" s="6">
-        <v>2026.0</v>
-      </c>
-      <c r="E11" s="6">
-        <v>6.0</v>
-      </c>
-      <c r="F11" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="B12" s="6">
-        <v>2003.0</v>
-      </c>
-      <c r="C12" s="6">
-        <v>8.0</v>
-      </c>
-      <c r="D12" s="6">
-        <v>2026.0</v>
-      </c>
-      <c r="E12" s="6">
-        <v>5.0</v>
-      </c>
-      <c r="F12" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="B13" s="6">
-        <v>2005.0</v>
-      </c>
-      <c r="C13" s="6">
-        <v>8.0</v>
-      </c>
-      <c r="D13" s="6">
-        <v>2026.0</v>
-      </c>
-      <c r="E13" s="6">
-        <v>10.0</v>
-      </c>
-      <c r="F13" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="B14" s="6">
-        <v>1997.0</v>
-      </c>
-      <c r="C14" s="6">
-        <v>8.0</v>
-      </c>
-      <c r="D14" s="6">
-        <v>2026.0</v>
-      </c>
-      <c r="E14" s="6">
-        <v>73.0</v>
-      </c>
-      <c r="F14" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="B15" s="6">
-        <v>2000.0</v>
-      </c>
-      <c r="C15" s="6">
-        <v>8.0</v>
-      </c>
-      <c r="D15" s="6">
-        <v>2026.0</v>
-      </c>
-      <c r="E15" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="F15" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="B16" s="6">
-        <v>1999.0</v>
-      </c>
-      <c r="C16" s="6">
-        <v>8.0</v>
-      </c>
-      <c r="D16" s="6">
-        <v>2026.0</v>
-      </c>
-      <c r="E16" s="6">
-        <v>218.0</v>
-      </c>
-      <c r="F16" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="B17" s="6">
-        <v>1999.0</v>
-      </c>
-      <c r="C17" s="6">
-        <v>9.0</v>
-      </c>
-      <c r="D17" s="6">
-        <v>2026.0</v>
-      </c>
-      <c r="E17" s="6">
-        <v>24.0</v>
-      </c>
-      <c r="F17" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="B18" s="6">
-        <v>1999.0</v>
-      </c>
-      <c r="C18" s="6">
-        <v>9.0</v>
-      </c>
-      <c r="D18" s="6">
-        <v>2026.0</v>
-      </c>
-      <c r="E18" s="6">
-        <v>13.0</v>
-      </c>
-      <c r="F18" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="B19" s="6">
-        <v>1998.0</v>
-      </c>
-      <c r="C19" s="6">
-        <v>9.0</v>
-      </c>
-      <c r="D19" s="6">
-        <v>2026.0</v>
-      </c>
-      <c r="E19" s="6">
-        <v>5.0</v>
-      </c>
-      <c r="F19" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="B20" s="6">
-        <v>2003.0</v>
-      </c>
-      <c r="C20" s="6">
-        <v>9.0</v>
-      </c>
-      <c r="D20" s="6">
-        <v>2026.0</v>
-      </c>
-      <c r="E20" s="6">
-        <v>35.0</v>
-      </c>
-      <c r="F20" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="B21" s="6">
-        <v>2003.0</v>
-      </c>
-      <c r="C21" s="6">
-        <v>9.0</v>
-      </c>
-      <c r="D21" s="6">
-        <v>2026.0</v>
-      </c>
-      <c r="E21" s="6">
-        <v>30.0</v>
-      </c>
-      <c r="F21" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="B22" s="6">
-        <v>2005.0</v>
-      </c>
-      <c r="C22" s="6">
-        <v>9.0</v>
-      </c>
-      <c r="D22" s="6">
-        <v>2026.0</v>
-      </c>
-      <c r="E22" s="6">
-        <v>45.0</v>
-      </c>
-      <c r="F22" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="B23" s="6">
-        <v>1999.0</v>
-      </c>
-      <c r="C23" s="6">
-        <v>6.0</v>
-      </c>
-      <c r="D23" s="6">
-        <v>2026.0</v>
-      </c>
-      <c r="E23" s="6">
-        <v>4.0</v>
-      </c>
-      <c r="F23" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="B24" s="7">
-        <v>2000.0</v>
-      </c>
-      <c r="C24" s="7">
-        <v>6.0</v>
-      </c>
-      <c r="D24" s="7">
-        <v>2026.0</v>
-      </c>
-      <c r="E24" s="7">
-        <v>27.0</v>
-      </c>
-      <c r="F24" s="7">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="B25" s="7">
-        <v>2000.0</v>
-      </c>
-      <c r="C25" s="7">
-        <v>6.0</v>
-      </c>
-      <c r="D25" s="7">
-        <v>2026.0</v>
-      </c>
-      <c r="E25" s="7">
-        <v>32.0</v>
-      </c>
-      <c r="F25" s="7">
-        <v>1.0</v>
-      </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="7" t="s">
+      <c r="A26" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="B26" s="7">
+      <c r="B26" s="3">
         <v>2002.0</v>
       </c>
       <c r="C26" s="8">
@@ -6287,7 +6279,7 @@
       <c r="D26" s="8">
         <v>2026.0</v>
       </c>
-      <c r="E26" s="7">
+      <c r="E26" s="3">
         <v>2.0</v>
       </c>
       <c r="F26" s="8">
@@ -6295,402 +6287,402 @@
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="7" t="s">
+      <c r="A27" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="B27" s="7">
+      <c r="B27" s="3">
         <v>1998.0</v>
       </c>
-      <c r="C27" s="7">
+      <c r="C27" s="3">
         <v>5.0</v>
       </c>
-      <c r="D27" s="7">
+      <c r="D27" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E27" s="7">
+      <c r="E27" s="3">
         <v>1.0</v>
       </c>
-      <c r="F27" s="7">
+      <c r="F27" s="3">
         <v>1.0</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="7" t="s">
+      <c r="A28" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="B28" s="7">
+      <c r="B28" s="3">
         <v>1995.0</v>
       </c>
-      <c r="C28" s="7">
+      <c r="C28" s="3">
         <v>5.0</v>
       </c>
-      <c r="D28" s="7">
+      <c r="D28" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E28" s="7">
+      <c r="E28" s="3">
         <v>21.0</v>
       </c>
-      <c r="F28" s="7">
+      <c r="F28" s="3">
         <v>1.0</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="7" t="s">
+      <c r="A29" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="B29" s="7">
+      <c r="B29" s="3">
         <v>1998.0</v>
       </c>
-      <c r="C29" s="7">
+      <c r="C29" s="3">
         <v>10.0</v>
       </c>
-      <c r="D29" s="7">
+      <c r="D29" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E29" s="7">
+      <c r="E29" s="3">
         <v>5.0</v>
       </c>
-      <c r="F29" s="7">
+      <c r="F29" s="3">
         <v>1.0</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="7" t="s">
+      <c r="A30" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="B30" s="7">
+      <c r="B30" s="3">
         <v>2000.0</v>
       </c>
-      <c r="C30" s="7">
+      <c r="C30" s="3">
         <v>10.0</v>
       </c>
-      <c r="D30" s="7">
+      <c r="D30" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E30" s="7">
+      <c r="E30" s="3">
         <v>20.0</v>
       </c>
-      <c r="F30" s="7">
+      <c r="F30" s="3">
         <v>1.0</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="7" t="s">
+      <c r="A31" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="B31" s="7">
+      <c r="B31" s="3">
         <v>2000.0</v>
       </c>
-      <c r="C31" s="7">
+      <c r="C31" s="3">
         <v>10.0</v>
       </c>
-      <c r="D31" s="7">
+      <c r="D31" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E31" s="7">
+      <c r="E31" s="3">
         <v>1.0</v>
       </c>
-      <c r="F31" s="7">
+      <c r="F31" s="3">
         <v>1.0</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="7" t="s">
+      <c r="A32" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="B32" s="7">
+      <c r="B32" s="3">
         <v>2003.0</v>
       </c>
-      <c r="C32" s="7">
+      <c r="C32" s="3">
         <v>10.0</v>
       </c>
-      <c r="D32" s="7">
+      <c r="D32" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E32" s="7">
+      <c r="E32" s="3">
         <v>1.0</v>
       </c>
-      <c r="F32" s="7">
+      <c r="F32" s="3">
         <v>1.0</v>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="7" t="s">
+      <c r="A33" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="B33" s="7">
+      <c r="B33" s="3">
         <v>1998.0</v>
       </c>
-      <c r="C33" s="7">
+      <c r="C33" s="3">
         <v>7.0</v>
       </c>
-      <c r="D33" s="7">
+      <c r="D33" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E33" s="7">
+      <c r="E33" s="3">
         <v>1.0</v>
       </c>
-      <c r="F33" s="7">
+      <c r="F33" s="3">
         <v>1.0</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="7" t="s">
+      <c r="A34" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="B34" s="7">
+      <c r="B34" s="3">
         <v>1999.0</v>
       </c>
-      <c r="C34" s="7">
+      <c r="C34" s="3">
         <v>7.0</v>
       </c>
-      <c r="D34" s="7">
+      <c r="D34" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E34" s="7">
+      <c r="E34" s="3">
         <v>6.0</v>
       </c>
-      <c r="F34" s="7">
+      <c r="F34" s="3">
         <v>1.0</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
-      <c r="A35" s="7" t="s">
+      <c r="A35" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="B35" s="7">
+      <c r="B35" s="3">
         <v>1999.0</v>
       </c>
-      <c r="C35" s="7">
+      <c r="C35" s="3">
         <v>7.0</v>
       </c>
-      <c r="D35" s="7">
+      <c r="D35" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E35" s="7">
+      <c r="E35" s="3">
         <v>35.0</v>
       </c>
-      <c r="F35" s="7">
+      <c r="F35" s="3">
         <v>1.0</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
-      <c r="A36" s="7" t="s">
+      <c r="A36" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="B36" s="7">
+      <c r="B36" s="3">
         <v>2005.0</v>
       </c>
-      <c r="C36" s="7">
+      <c r="C36" s="3">
         <v>7.0</v>
       </c>
-      <c r="D36" s="7">
+      <c r="D36" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E36" s="7">
+      <c r="E36" s="3">
         <v>7.0</v>
       </c>
-      <c r="F36" s="7">
+      <c r="F36" s="3">
         <v>1.0</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
-      <c r="A37" s="7" t="s">
+      <c r="A37" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="B37" s="7">
+      <c r="B37" s="3">
         <v>2000.0</v>
       </c>
-      <c r="C37" s="7">
+      <c r="C37" s="3">
         <v>2.0</v>
       </c>
-      <c r="D37" s="7">
+      <c r="D37" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E37" s="7">
+      <c r="E37" s="3">
         <v>92.0</v>
       </c>
-      <c r="F37" s="7">
+      <c r="F37" s="3">
         <v>1.0</v>
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="7" t="s">
+      <c r="A38" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="B38" s="7">
+      <c r="B38" s="3">
         <v>2003.0</v>
       </c>
-      <c r="C38" s="7">
+      <c r="C38" s="3">
         <v>2.0</v>
       </c>
-      <c r="D38" s="7">
+      <c r="D38" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E38" s="7">
+      <c r="E38" s="3">
         <v>50.0</v>
       </c>
-      <c r="F38" s="7">
+      <c r="F38" s="3">
         <v>1.0</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
-      <c r="A39" s="7" t="s">
+      <c r="A39" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="B39" s="7">
+      <c r="B39" s="3">
         <v>1994.0</v>
       </c>
-      <c r="C39" s="7">
+      <c r="C39" s="3">
         <v>2.0</v>
       </c>
-      <c r="D39" s="7">
+      <c r="D39" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E39" s="7">
+      <c r="E39" s="3">
         <v>25.0</v>
       </c>
-      <c r="F39" s="7">
+      <c r="F39" s="3">
         <v>1.0</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
-      <c r="A40" s="7" t="s">
+      <c r="A40" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="B40" s="3">
+        <v>2004.0</v>
+      </c>
+      <c r="C40" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="D40" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="E40" s="3">
+        <v>5.0</v>
+      </c>
+      <c r="F40" s="3">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="41" ht="15.75" customHeight="1">
+      <c r="A41" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="B40" s="7">
-        <v>2004.0</v>
-      </c>
-      <c r="C40" s="7">
+      <c r="B41" s="3">
+        <v>2002.0</v>
+      </c>
+      <c r="C41" s="3">
         <v>2.0</v>
       </c>
-      <c r="D40" s="7">
+      <c r="D41" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E40" s="7">
-        <v>5.0</v>
-      </c>
-      <c r="F40" s="7">
+      <c r="E41" s="3">
+        <v>31.0</v>
+      </c>
+      <c r="F41" s="3">
         <v>1.0</v>
       </c>
     </row>
-    <row r="41" ht="15.75" customHeight="1">
-      <c r="A41" s="7" t="s">
+    <row r="42" ht="15.75" customHeight="1">
+      <c r="A42" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="B41" s="7">
-        <v>2002.0</v>
-      </c>
-      <c r="C41" s="7">
+      <c r="B42" s="3">
+        <v>1995.0</v>
+      </c>
+      <c r="C42" s="3">
         <v>2.0</v>
       </c>
-      <c r="D41" s="7">
+      <c r="D42" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E41" s="7">
+      <c r="E42" s="3">
+        <v>42.0</v>
+      </c>
+      <c r="F42" s="3">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="43" ht="15.75" customHeight="1">
+      <c r="A43" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="B43" s="3">
+        <v>1996.0</v>
+      </c>
+      <c r="C43" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="D43" s="3">
+        <v>2026.0</v>
+      </c>
+      <c r="E43" s="3">
         <v>31.0</v>
       </c>
-      <c r="F41" s="7">
+      <c r="F43" s="3">
         <v>1.0</v>
       </c>
     </row>
-    <row r="42" ht="15.75" customHeight="1">
-      <c r="A42" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="B42" s="7">
-        <v>1995.0</v>
-      </c>
-      <c r="C42" s="7">
-        <v>2.0</v>
-      </c>
-      <c r="D42" s="7">
+    <row r="44" ht="15.75" customHeight="1">
+      <c r="A44" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="B44" s="3">
+        <v>2003.0</v>
+      </c>
+      <c r="C44" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="D44" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E42" s="7">
-        <v>42.0</v>
-      </c>
-      <c r="F42" s="7">
+      <c r="E44" s="3">
+        <v>11.0</v>
+      </c>
+      <c r="F44" s="3">
         <v>1.0</v>
       </c>
     </row>
-    <row r="43" ht="15.75" customHeight="1">
-      <c r="A43" s="7" t="s">
-        <v>141</v>
-      </c>
-      <c r="B43" s="7">
-        <v>1996.0</v>
-      </c>
-      <c r="C43" s="7">
+    <row r="45" ht="15.75" customHeight="1">
+      <c r="A45" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="B45" s="3">
+        <v>2001.0</v>
+      </c>
+      <c r="C45" s="3">
         <v>1.0</v>
       </c>
-      <c r="D43" s="7">
+      <c r="D45" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E43" s="7">
-        <v>31.0</v>
-      </c>
-      <c r="F43" s="7">
+      <c r="E45" s="3">
         <v>1.0</v>
       </c>
-    </row>
-    <row r="44" ht="15.75" customHeight="1">
-      <c r="A44" s="7" t="s">
-        <v>142</v>
-      </c>
-      <c r="B44" s="7">
-        <v>2003.0</v>
-      </c>
-      <c r="C44" s="7">
+      <c r="F45" s="3">
         <v>1.0</v>
       </c>
-      <c r="D44" s="7">
+    </row>
+    <row r="46" ht="15.75" customHeight="1">
+      <c r="A46" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="B46" s="3">
+        <v>1997.0</v>
+      </c>
+      <c r="C46" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="D46" s="3">
         <v>2026.0</v>
       </c>
-      <c r="E44" s="7">
-        <v>11.0</v>
-      </c>
-      <c r="F44" s="7">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="45" ht="15.75" customHeight="1">
-      <c r="A45" s="7" t="s">
-        <v>143</v>
-      </c>
-      <c r="B45" s="7">
-        <v>2001.0</v>
-      </c>
-      <c r="C45" s="7">
-        <v>1.0</v>
-      </c>
-      <c r="D45" s="7">
-        <v>2026.0</v>
-      </c>
-      <c r="E45" s="7">
-        <v>1.0</v>
-      </c>
-      <c r="F45" s="7">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="46" ht="15.75" customHeight="1">
-      <c r="A46" s="7" t="s">
-        <v>144</v>
-      </c>
-      <c r="B46" s="7">
-        <v>1997.0</v>
-      </c>
-      <c r="C46" s="7">
-        <v>1.0</v>
-      </c>
-      <c r="D46" s="7">
-        <v>2026.0</v>
-      </c>
-      <c r="E46" s="7">
+      <c r="E46" s="3">
         <v>24.0</v>
       </c>
-      <c r="F46" s="7">
+      <c r="F46" s="3">
         <v>1.0</v>
       </c>
     </row>
@@ -7671,20 +7663,20 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="B1" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="C1" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="D1" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="E1" s="9" t="s">
-        <v>77</v>
+      <c r="A1" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -8692,23 +8684,23 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="2" t="s">
+      <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="C1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>6</v>
+      <c r="E1" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="2">
@@ -8728,7 +8720,7 @@
         <v>1.0</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>62</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3">
@@ -8748,7 +8740,7 @@
         <v>0.0</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>52</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4">
@@ -8768,7 +8760,7 @@
         <v>0.0</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>48</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5">
@@ -8788,7 +8780,7 @@
         <v>0.0</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>64</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6">
@@ -8808,7 +8800,7 @@
         <v>0.0</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>59</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7">
@@ -8828,7 +8820,7 @@
         <v>0.0</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8">
@@ -8848,7 +8840,7 @@
         <v>0.0</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>37</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
@@ -8868,7 +8860,7 @@
         <v>0.0</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>67</v>
+        <v>41</v>
       </c>
     </row>
     <row r="10">
@@ -8888,7 +8880,7 @@
         <v>0.0</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>41</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11">
@@ -8908,7 +8900,7 @@
         <v>0.0</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>55</v>
+        <v>23</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -9914,17 +9906,17 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>6</v>
+      <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="2">
@@ -9938,7 +9930,7 @@
         <v>4.0</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>48</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3">
@@ -9952,7 +9944,7 @@
         <v>8.0</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>62</v>
+        <v>31</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -10957,17 +10949,17 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>31</v>
+      <c r="D1" s="1" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="2">
@@ -10981,7 +10973,7 @@
         <v>32.0</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>33</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
@@ -10995,7 +10987,7 @@
         <v>13.0</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>39</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
@@ -11009,7 +11001,7 @@
         <v>34.0</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>47</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5">
@@ -11023,7 +11015,7 @@
         <v>10.0</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>54</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6">
@@ -11037,7 +11029,7 @@
         <v>1.0</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>58</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7">
@@ -11051,7 +11043,7 @@
         <v>4.0</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>66</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8">
@@ -11065,7 +11057,7 @@
         <v>33.0</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>71</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9">
@@ -11079,7 +11071,7 @@
         <v>13.0</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>76</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10">
@@ -11093,7 +11085,7 @@
         <v>14.0</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>81</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11">
@@ -11107,7 +11099,7 @@
         <v>27.0</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>85</v>
+        <v>39</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -12115,25 +12107,25 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D1" s="2" t="s">
+      <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>149</v>
       </c>
     </row>
@@ -12145,7 +12137,7 @@
         <v>1.0</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>37</v>
+        <v>8</v>
       </c>
       <c r="D2" s="3">
         <v>-5.0</v>
@@ -12168,7 +12160,7 @@
         <v>2.0</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="D3" s="3">
         <v>-15.0</v>
@@ -12191,7 +12183,7 @@
         <v>3.0</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="D4" s="3">
         <v>0.0</v>
@@ -12214,7 +12206,7 @@
         <v>4.0</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>48</v>
+        <v>16</v>
       </c>
       <c r="D5" s="3">
         <v>10.0</v>
@@ -12237,7 +12229,7 @@
         <v>5.0</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>52</v>
+        <v>19</v>
       </c>
       <c r="D6" s="3">
         <v>15.0</v>
@@ -12260,7 +12252,7 @@
         <v>6.0</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>55</v>
+        <v>23</v>
       </c>
       <c r="D7" s="3">
         <v>-20.0</v>
@@ -12283,7 +12275,7 @@
         <v>7.0</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>59</v>
+        <v>26</v>
       </c>
       <c r="D8" s="3">
         <v>0.0</v>
@@ -12306,7 +12298,7 @@
         <v>8.0</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>62</v>
+        <v>31</v>
       </c>
       <c r="D9" s="3">
         <v>25.0</v>
@@ -12329,7 +12321,7 @@
         <v>9.0</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>64</v>
+        <v>36</v>
       </c>
       <c r="D10" s="3">
         <v>5.0</v>
@@ -12352,7 +12344,7 @@
         <v>10.0</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>67</v>
+        <v>41</v>
       </c>
       <c r="D11" s="3">
         <v>-10.0</v>

</xml_diff>